<commit_message>
feat: save system, club feedback mails, game-feel effects, resume salary/career
- Easy Save 3 integration: versioned WeekStateSnapshot in Domain, JSON
  snapshot in new Persistence assembly, autosave on end-week, restore on
  launch, restart deletes save; seeded random restored via draw count
- Club feedback mails: qualitative multi-tier evaluations 1-2 weeks after
  placement, stable IDs, regenerated from delivered outcomes on load
- Game feel: end-week black fade with date card, workspace crossfade,
  click punch; pacing tuned for a thinking game
- Fix portrait/text overlap: container-anchored 1:1 RawImage structure
  for player cards, resume portraits and magazine covers
- Player resume: public weekly salary range + career history for all
  16 players; submission template and tests updated
- Enable Easy Save 3 asmdefs; scene rebuilt via builder menu command

EditMode 29/29, PlayMode 5/5
</commit_message>
<xml_diff>
--- a/output/spreadsheet/NewPlayerHunter_Content_Submission_Template.xlsx
+++ b/output/spreadsheet/NewPlayerHunter_Content_Submission_Template.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="球员 Players" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招聘 Demands" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招聘槽位 DemandSlots" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="邮件 Mails" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="期刊 Issues" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="期刊页面 MagazinePages" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附件 Assets" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交检查" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="使用说明" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="球员 Players" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="招聘 Demands" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="招聘槽位 DemandSlots" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="邮件 Mails" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="期刊 Issues" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="期刊页面 MagazinePages" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="附件 Assets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="提交检查" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'球员 Players'!$A$4:$S$205</definedName>
@@ -275,47 +275,47 @@
         <t>必填。隐藏职业性 0–100</t>
       </text>
     </comment>
-    <comment ref="K4" authorId="0" shapeId="0">
+    <comment ref="O4" authorId="0" shapeId="0">
       <text>
         <t>必填。本人、经纪人或亲友的公开声明</t>
       </text>
     </comment>
-    <comment ref="L4" authorId="0" shapeId="0">
+    <comment ref="P4" authorId="0" shapeId="0">
       <text>
         <t>可选。英文公开声明</t>
       </text>
     </comment>
-    <comment ref="M4" authorId="0" shapeId="0">
+    <comment ref="Q4" authorId="0" shapeId="0">
       <text>
         <t>必填。公开旁证或交叉信息</t>
       </text>
     </comment>
-    <comment ref="N4" authorId="0" shapeId="0">
+    <comment ref="R4" authorId="0" shapeId="0">
       <text>
         <t>可选。英文旁证</t>
       </text>
     </comment>
-    <comment ref="O4" authorId="0" shapeId="0">
+    <comment ref="S4" authorId="0" shapeId="0">
       <text>
         <t>必填。公开证据可靠性枚举</t>
       </text>
     </comment>
-    <comment ref="P4" authorId="0" shapeId="0">
+    <comment ref="T4" authorId="0" shapeId="0">
       <text>
         <t>可选。仅给编辑看的原型和笑点说明，不进入游戏</t>
       </text>
     </comment>
-    <comment ref="Q4" authorId="0" shapeId="0">
+    <comment ref="U4" authorId="0" shapeId="0">
       <text>
         <t>可选。原创肖像构图、服装、表情和禁止元素</t>
       </text>
     </comment>
-    <comment ref="R4" authorId="0" shapeId="0">
+    <comment ref="V4" authorId="0" shapeId="0">
       <text>
         <t>可选。对应附件文件名</t>
       </text>
     </comment>
-    <comment ref="S4" authorId="0" shapeId="0">
+    <comment ref="W4" authorId="0" shapeId="0">
       <text>
         <t>可选。给整合人员的备注</t>
       </text>
@@ -1269,7 +1269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S205"/>
+  <dimension ref="A1:W205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1307,6 +1307,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -1360,45 +1361,65 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>public_claim_zh</t>
+          <t>salary_min_weekly</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>public_claim_en</t>
+          <t>salary_max_weekly</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>public_evidence_zh</t>
+          <t>career_history_zh</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>public_evidence_en</t>
+          <t>career_history_en</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>evidence_reliability</t>
+          <t>public_claim_zh</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>inspiration_notes_private</t>
+          <t>public_claim_en</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
-          <t>portrait_brief</t>
+          <t>public_evidence_zh</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr">
         <is>
+          <t>public_evidence_en</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>evidence_reliability</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>inspiration_notes_private</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>portrait_brief</t>
+        </is>
+      </c>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
           <t>asset_filename</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="W4" s="5" t="inlineStr">
         <is>
           <t>integrator_notes</t>
         </is>
@@ -1441,27 +1462,27 @@
       <c r="J5" s="6" t="n">
         <v>61</v>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>经纪人声称他能追上自己昨天的传球。</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr"/>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="P5" s="6" t="inlineStr"/>
+      <c r="Q5" s="6" t="inlineStr">
         <is>
           <t>两场录像确认速度不错，但触球稳定性存疑。</t>
         </is>
       </c>
-      <c r="N5" s="6" t="inlineStr"/>
-      <c r="O5" s="6" t="inlineStr">
+      <c r="R5" s="6" t="inlineStr"/>
+      <c r="S5" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P5" s="6" t="inlineStr"/>
-      <c r="Q5" s="6" t="inlineStr"/>
-      <c r="R5" s="6" t="inlineStr"/>
-      <c r="S5" s="6" t="inlineStr">
+      <c r="T5" s="6" t="inlineStr"/>
+      <c r="U5" s="6" t="inlineStr"/>
+      <c r="V5" s="6" t="inlineStr"/>
+      <c r="W5" s="6" t="inlineStr">
         <is>
           <t>示例行，请勿直接提交。</t>
         </is>
@@ -1478,15 +1499,15 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="7" t="n"/>
-      <c r="N6" s="7" t="n"/>
       <c r="O6" s="7" t="n"/>
       <c r="P6" s="7" t="n"/>
       <c r="Q6" s="7" t="n"/>
       <c r="R6" s="7" t="n"/>
       <c r="S6" s="7" t="n"/>
+      <c r="T6" s="7" t="n"/>
+      <c r="U6" s="7" t="n"/>
+      <c r="V6" s="7" t="n"/>
+      <c r="W6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n"/>
@@ -1499,15 +1520,15 @@
       <c r="H7" s="7" t="n"/>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
       <c r="O7" s="7" t="n"/>
       <c r="P7" s="7" t="n"/>
       <c r="Q7" s="7" t="n"/>
       <c r="R7" s="7" t="n"/>
       <c r="S7" s="7" t="n"/>
+      <c r="T7" s="7" t="n"/>
+      <c r="U7" s="7" t="n"/>
+      <c r="V7" s="7" t="n"/>
+      <c r="W7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n"/>
@@ -1520,15 +1541,15 @@
       <c r="H8" s="7" t="n"/>
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
       <c r="O8" s="7" t="n"/>
       <c r="P8" s="7" t="n"/>
       <c r="Q8" s="7" t="n"/>
       <c r="R8" s="7" t="n"/>
       <c r="S8" s="7" t="n"/>
+      <c r="T8" s="7" t="n"/>
+      <c r="U8" s="7" t="n"/>
+      <c r="V8" s="7" t="n"/>
+      <c r="W8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
@@ -1541,15 +1562,15 @@
       <c r="H9" s="7" t="n"/>
       <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
       <c r="O9" s="7" t="n"/>
       <c r="P9" s="7" t="n"/>
       <c r="Q9" s="7" t="n"/>
       <c r="R9" s="7" t="n"/>
       <c r="S9" s="7" t="n"/>
+      <c r="T9" s="7" t="n"/>
+      <c r="U9" s="7" t="n"/>
+      <c r="V9" s="7" t="n"/>
+      <c r="W9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
@@ -1562,15 +1583,15 @@
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="n"/>
-      <c r="K10" s="7" t="n"/>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="n"/>
-      <c r="N10" s="7" t="n"/>
       <c r="O10" s="7" t="n"/>
       <c r="P10" s="7" t="n"/>
       <c r="Q10" s="7" t="n"/>
       <c r="R10" s="7" t="n"/>
       <c r="S10" s="7" t="n"/>
+      <c r="T10" s="7" t="n"/>
+      <c r="U10" s="7" t="n"/>
+      <c r="V10" s="7" t="n"/>
+      <c r="W10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -1583,15 +1604,15 @@
       <c r="H11" s="7" t="n"/>
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="n"/>
-      <c r="N11" s="7" t="n"/>
       <c r="O11" s="7" t="n"/>
       <c r="P11" s="7" t="n"/>
       <c r="Q11" s="7" t="n"/>
       <c r="R11" s="7" t="n"/>
       <c r="S11" s="7" t="n"/>
+      <c r="T11" s="7" t="n"/>
+      <c r="U11" s="7" t="n"/>
+      <c r="V11" s="7" t="n"/>
+      <c r="W11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -1604,15 +1625,15 @@
       <c r="H12" s="7" t="n"/>
       <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="n"/>
-      <c r="K12" s="7" t="n"/>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7" t="n"/>
-      <c r="N12" s="7" t="n"/>
       <c r="O12" s="7" t="n"/>
       <c r="P12" s="7" t="n"/>
       <c r="Q12" s="7" t="n"/>
       <c r="R12" s="7" t="n"/>
       <c r="S12" s="7" t="n"/>
+      <c r="T12" s="7" t="n"/>
+      <c r="U12" s="7" t="n"/>
+      <c r="V12" s="7" t="n"/>
+      <c r="W12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -1625,15 +1646,15 @@
       <c r="H13" s="7" t="n"/>
       <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="n"/>
-      <c r="K13" s="7" t="n"/>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="n"/>
-      <c r="N13" s="7" t="n"/>
       <c r="O13" s="7" t="n"/>
       <c r="P13" s="7" t="n"/>
       <c r="Q13" s="7" t="n"/>
       <c r="R13" s="7" t="n"/>
       <c r="S13" s="7" t="n"/>
+      <c r="T13" s="7" t="n"/>
+      <c r="U13" s="7" t="n"/>
+      <c r="V13" s="7" t="n"/>
+      <c r="W13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -1646,15 +1667,15 @@
       <c r="H14" s="7" t="n"/>
       <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="n"/>
-      <c r="K14" s="7" t="n"/>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7" t="n"/>
-      <c r="N14" s="7" t="n"/>
       <c r="O14" s="7" t="n"/>
       <c r="P14" s="7" t="n"/>
       <c r="Q14" s="7" t="n"/>
       <c r="R14" s="7" t="n"/>
       <c r="S14" s="7" t="n"/>
+      <c r="T14" s="7" t="n"/>
+      <c r="U14" s="7" t="n"/>
+      <c r="V14" s="7" t="n"/>
+      <c r="W14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -1667,15 +1688,15 @@
       <c r="H15" s="7" t="n"/>
       <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="n"/>
-      <c r="K15" s="7" t="n"/>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7" t="n"/>
-      <c r="N15" s="7" t="n"/>
       <c r="O15" s="7" t="n"/>
       <c r="P15" s="7" t="n"/>
       <c r="Q15" s="7" t="n"/>
       <c r="R15" s="7" t="n"/>
       <c r="S15" s="7" t="n"/>
+      <c r="T15" s="7" t="n"/>
+      <c r="U15" s="7" t="n"/>
+      <c r="V15" s="7" t="n"/>
+      <c r="W15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -1688,15 +1709,15 @@
       <c r="H16" s="7" t="n"/>
       <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="n"/>
-      <c r="K16" s="7" t="n"/>
-      <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7" t="n"/>
-      <c r="N16" s="7" t="n"/>
       <c r="O16" s="7" t="n"/>
       <c r="P16" s="7" t="n"/>
       <c r="Q16" s="7" t="n"/>
       <c r="R16" s="7" t="n"/>
       <c r="S16" s="7" t="n"/>
+      <c r="T16" s="7" t="n"/>
+      <c r="U16" s="7" t="n"/>
+      <c r="V16" s="7" t="n"/>
+      <c r="W16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -1709,15 +1730,15 @@
       <c r="H17" s="7" t="n"/>
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
-      <c r="M17" s="7" t="n"/>
-      <c r="N17" s="7" t="n"/>
       <c r="O17" s="7" t="n"/>
       <c r="P17" s="7" t="n"/>
       <c r="Q17" s="7" t="n"/>
       <c r="R17" s="7" t="n"/>
       <c r="S17" s="7" t="n"/>
+      <c r="T17" s="7" t="n"/>
+      <c r="U17" s="7" t="n"/>
+      <c r="V17" s="7" t="n"/>
+      <c r="W17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -1730,15 +1751,15 @@
       <c r="H18" s="7" t="n"/>
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
-      <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
-      <c r="M18" s="7" t="n"/>
-      <c r="N18" s="7" t="n"/>
       <c r="O18" s="7" t="n"/>
       <c r="P18" s="7" t="n"/>
       <c r="Q18" s="7" t="n"/>
       <c r="R18" s="7" t="n"/>
       <c r="S18" s="7" t="n"/>
+      <c r="T18" s="7" t="n"/>
+      <c r="U18" s="7" t="n"/>
+      <c r="V18" s="7" t="n"/>
+      <c r="W18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -1751,15 +1772,15 @@
       <c r="H19" s="7" t="n"/>
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
-      <c r="K19" s="7" t="n"/>
-      <c r="L19" s="7" t="n"/>
-      <c r="M19" s="7" t="n"/>
-      <c r="N19" s="7" t="n"/>
       <c r="O19" s="7" t="n"/>
       <c r="P19" s="7" t="n"/>
       <c r="Q19" s="7" t="n"/>
       <c r="R19" s="7" t="n"/>
       <c r="S19" s="7" t="n"/>
+      <c r="T19" s="7" t="n"/>
+      <c r="U19" s="7" t="n"/>
+      <c r="V19" s="7" t="n"/>
+      <c r="W19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -1772,15 +1793,15 @@
       <c r="H20" s="7" t="n"/>
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="n"/>
-      <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
-      <c r="N20" s="7" t="n"/>
       <c r="O20" s="7" t="n"/>
       <c r="P20" s="7" t="n"/>
       <c r="Q20" s="7" t="n"/>
       <c r="R20" s="7" t="n"/>
       <c r="S20" s="7" t="n"/>
+      <c r="T20" s="7" t="n"/>
+      <c r="U20" s="7" t="n"/>
+      <c r="V20" s="7" t="n"/>
+      <c r="W20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
@@ -1793,15 +1814,15 @@
       <c r="H21" s="7" t="n"/>
       <c r="I21" s="7" t="n"/>
       <c r="J21" s="7" t="n"/>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
       <c r="O21" s="7" t="n"/>
       <c r="P21" s="7" t="n"/>
       <c r="Q21" s="7" t="n"/>
       <c r="R21" s="7" t="n"/>
       <c r="S21" s="7" t="n"/>
+      <c r="T21" s="7" t="n"/>
+      <c r="U21" s="7" t="n"/>
+      <c r="V21" s="7" t="n"/>
+      <c r="W21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
@@ -1814,15 +1835,15 @@
       <c r="H22" s="7" t="n"/>
       <c r="I22" s="7" t="n"/>
       <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
-      <c r="N22" s="7" t="n"/>
       <c r="O22" s="7" t="n"/>
       <c r="P22" s="7" t="n"/>
       <c r="Q22" s="7" t="n"/>
       <c r="R22" s="7" t="n"/>
       <c r="S22" s="7" t="n"/>
+      <c r="T22" s="7" t="n"/>
+      <c r="U22" s="7" t="n"/>
+      <c r="V22" s="7" t="n"/>
+      <c r="W22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -1835,15 +1856,15 @@
       <c r="H23" s="7" t="n"/>
       <c r="I23" s="7" t="n"/>
       <c r="J23" s="7" t="n"/>
-      <c r="K23" s="7" t="n"/>
-      <c r="L23" s="7" t="n"/>
-      <c r="M23" s="7" t="n"/>
-      <c r="N23" s="7" t="n"/>
       <c r="O23" s="7" t="n"/>
       <c r="P23" s="7" t="n"/>
       <c r="Q23" s="7" t="n"/>
       <c r="R23" s="7" t="n"/>
       <c r="S23" s="7" t="n"/>
+      <c r="T23" s="7" t="n"/>
+      <c r="U23" s="7" t="n"/>
+      <c r="V23" s="7" t="n"/>
+      <c r="W23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
@@ -1856,15 +1877,15 @@
       <c r="H24" s="7" t="n"/>
       <c r="I24" s="7" t="n"/>
       <c r="J24" s="7" t="n"/>
-      <c r="K24" s="7" t="n"/>
-      <c r="L24" s="7" t="n"/>
-      <c r="M24" s="7" t="n"/>
-      <c r="N24" s="7" t="n"/>
       <c r="O24" s="7" t="n"/>
       <c r="P24" s="7" t="n"/>
       <c r="Q24" s="7" t="n"/>
       <c r="R24" s="7" t="n"/>
       <c r="S24" s="7" t="n"/>
+      <c r="T24" s="7" t="n"/>
+      <c r="U24" s="7" t="n"/>
+      <c r="V24" s="7" t="n"/>
+      <c r="W24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -1877,15 +1898,15 @@
       <c r="H25" s="7" t="n"/>
       <c r="I25" s="7" t="n"/>
       <c r="J25" s="7" t="n"/>
-      <c r="K25" s="7" t="n"/>
-      <c r="L25" s="7" t="n"/>
-      <c r="M25" s="7" t="n"/>
-      <c r="N25" s="7" t="n"/>
       <c r="O25" s="7" t="n"/>
       <c r="P25" s="7" t="n"/>
       <c r="Q25" s="7" t="n"/>
       <c r="R25" s="7" t="n"/>
       <c r="S25" s="7" t="n"/>
+      <c r="T25" s="7" t="n"/>
+      <c r="U25" s="7" t="n"/>
+      <c r="V25" s="7" t="n"/>
+      <c r="W25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -1898,15 +1919,15 @@
       <c r="H26" s="7" t="n"/>
       <c r="I26" s="7" t="n"/>
       <c r="J26" s="7" t="n"/>
-      <c r="K26" s="7" t="n"/>
-      <c r="L26" s="7" t="n"/>
-      <c r="M26" s="7" t="n"/>
-      <c r="N26" s="7" t="n"/>
       <c r="O26" s="7" t="n"/>
       <c r="P26" s="7" t="n"/>
       <c r="Q26" s="7" t="n"/>
       <c r="R26" s="7" t="n"/>
       <c r="S26" s="7" t="n"/>
+      <c r="T26" s="7" t="n"/>
+      <c r="U26" s="7" t="n"/>
+      <c r="V26" s="7" t="n"/>
+      <c r="W26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
@@ -1919,15 +1940,15 @@
       <c r="H27" s="7" t="n"/>
       <c r="I27" s="7" t="n"/>
       <c r="J27" s="7" t="n"/>
-      <c r="K27" s="7" t="n"/>
-      <c r="L27" s="7" t="n"/>
-      <c r="M27" s="7" t="n"/>
-      <c r="N27" s="7" t="n"/>
       <c r="O27" s="7" t="n"/>
       <c r="P27" s="7" t="n"/>
       <c r="Q27" s="7" t="n"/>
       <c r="R27" s="7" t="n"/>
       <c r="S27" s="7" t="n"/>
+      <c r="T27" s="7" t="n"/>
+      <c r="U27" s="7" t="n"/>
+      <c r="V27" s="7" t="n"/>
+      <c r="W27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
@@ -1940,15 +1961,15 @@
       <c r="H28" s="7" t="n"/>
       <c r="I28" s="7" t="n"/>
       <c r="J28" s="7" t="n"/>
-      <c r="K28" s="7" t="n"/>
-      <c r="L28" s="7" t="n"/>
-      <c r="M28" s="7" t="n"/>
-      <c r="N28" s="7" t="n"/>
       <c r="O28" s="7" t="n"/>
       <c r="P28" s="7" t="n"/>
       <c r="Q28" s="7" t="n"/>
       <c r="R28" s="7" t="n"/>
       <c r="S28" s="7" t="n"/>
+      <c r="T28" s="7" t="n"/>
+      <c r="U28" s="7" t="n"/>
+      <c r="V28" s="7" t="n"/>
+      <c r="W28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -1961,15 +1982,15 @@
       <c r="H29" s="7" t="n"/>
       <c r="I29" s="7" t="n"/>
       <c r="J29" s="7" t="n"/>
-      <c r="K29" s="7" t="n"/>
-      <c r="L29" s="7" t="n"/>
-      <c r="M29" s="7" t="n"/>
-      <c r="N29" s="7" t="n"/>
       <c r="O29" s="7" t="n"/>
       <c r="P29" s="7" t="n"/>
       <c r="Q29" s="7" t="n"/>
       <c r="R29" s="7" t="n"/>
       <c r="S29" s="7" t="n"/>
+      <c r="T29" s="7" t="n"/>
+      <c r="U29" s="7" t="n"/>
+      <c r="V29" s="7" t="n"/>
+      <c r="W29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
@@ -1982,15 +2003,15 @@
       <c r="H30" s="7" t="n"/>
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="7" t="n"/>
-      <c r="K30" s="7" t="n"/>
-      <c r="L30" s="7" t="n"/>
-      <c r="M30" s="7" t="n"/>
-      <c r="N30" s="7" t="n"/>
       <c r="O30" s="7" t="n"/>
       <c r="P30" s="7" t="n"/>
       <c r="Q30" s="7" t="n"/>
       <c r="R30" s="7" t="n"/>
       <c r="S30" s="7" t="n"/>
+      <c r="T30" s="7" t="n"/>
+      <c r="U30" s="7" t="n"/>
+      <c r="V30" s="7" t="n"/>
+      <c r="W30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
@@ -2003,15 +2024,15 @@
       <c r="H31" s="7" t="n"/>
       <c r="I31" s="7" t="n"/>
       <c r="J31" s="7" t="n"/>
-      <c r="K31" s="7" t="n"/>
-      <c r="L31" s="7" t="n"/>
-      <c r="M31" s="7" t="n"/>
-      <c r="N31" s="7" t="n"/>
       <c r="O31" s="7" t="n"/>
       <c r="P31" s="7" t="n"/>
       <c r="Q31" s="7" t="n"/>
       <c r="R31" s="7" t="n"/>
       <c r="S31" s="7" t="n"/>
+      <c r="T31" s="7" t="n"/>
+      <c r="U31" s="7" t="n"/>
+      <c r="V31" s="7" t="n"/>
+      <c r="W31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
@@ -2024,15 +2045,15 @@
       <c r="H32" s="7" t="n"/>
       <c r="I32" s="7" t="n"/>
       <c r="J32" s="7" t="n"/>
-      <c r="K32" s="7" t="n"/>
-      <c r="L32" s="7" t="n"/>
-      <c r="M32" s="7" t="n"/>
-      <c r="N32" s="7" t="n"/>
       <c r="O32" s="7" t="n"/>
       <c r="P32" s="7" t="n"/>
       <c r="Q32" s="7" t="n"/>
       <c r="R32" s="7" t="n"/>
       <c r="S32" s="7" t="n"/>
+      <c r="T32" s="7" t="n"/>
+      <c r="U32" s="7" t="n"/>
+      <c r="V32" s="7" t="n"/>
+      <c r="W32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
@@ -2045,15 +2066,15 @@
       <c r="H33" s="7" t="n"/>
       <c r="I33" s="7" t="n"/>
       <c r="J33" s="7" t="n"/>
-      <c r="K33" s="7" t="n"/>
-      <c r="L33" s="7" t="n"/>
-      <c r="M33" s="7" t="n"/>
-      <c r="N33" s="7" t="n"/>
       <c r="O33" s="7" t="n"/>
       <c r="P33" s="7" t="n"/>
       <c r="Q33" s="7" t="n"/>
       <c r="R33" s="7" t="n"/>
       <c r="S33" s="7" t="n"/>
+      <c r="T33" s="7" t="n"/>
+      <c r="U33" s="7" t="n"/>
+      <c r="V33" s="7" t="n"/>
+      <c r="W33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n"/>
@@ -2066,15 +2087,15 @@
       <c r="H34" s="7" t="n"/>
       <c r="I34" s="7" t="n"/>
       <c r="J34" s="7" t="n"/>
-      <c r="K34" s="7" t="n"/>
-      <c r="L34" s="7" t="n"/>
-      <c r="M34" s="7" t="n"/>
-      <c r="N34" s="7" t="n"/>
       <c r="O34" s="7" t="n"/>
       <c r="P34" s="7" t="n"/>
       <c r="Q34" s="7" t="n"/>
       <c r="R34" s="7" t="n"/>
       <c r="S34" s="7" t="n"/>
+      <c r="T34" s="7" t="n"/>
+      <c r="U34" s="7" t="n"/>
+      <c r="V34" s="7" t="n"/>
+      <c r="W34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n"/>
@@ -2087,15 +2108,15 @@
       <c r="H35" s="7" t="n"/>
       <c r="I35" s="7" t="n"/>
       <c r="J35" s="7" t="n"/>
-      <c r="K35" s="7" t="n"/>
-      <c r="L35" s="7" t="n"/>
-      <c r="M35" s="7" t="n"/>
-      <c r="N35" s="7" t="n"/>
       <c r="O35" s="7" t="n"/>
       <c r="P35" s="7" t="n"/>
       <c r="Q35" s="7" t="n"/>
       <c r="R35" s="7" t="n"/>
       <c r="S35" s="7" t="n"/>
+      <c r="T35" s="7" t="n"/>
+      <c r="U35" s="7" t="n"/>
+      <c r="V35" s="7" t="n"/>
+      <c r="W35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
@@ -2108,15 +2129,15 @@
       <c r="H36" s="7" t="n"/>
       <c r="I36" s="7" t="n"/>
       <c r="J36" s="7" t="n"/>
-      <c r="K36" s="7" t="n"/>
-      <c r="L36" s="7" t="n"/>
-      <c r="M36" s="7" t="n"/>
-      <c r="N36" s="7" t="n"/>
       <c r="O36" s="7" t="n"/>
       <c r="P36" s="7" t="n"/>
       <c r="Q36" s="7" t="n"/>
       <c r="R36" s="7" t="n"/>
       <c r="S36" s="7" t="n"/>
+      <c r="T36" s="7" t="n"/>
+      <c r="U36" s="7" t="n"/>
+      <c r="V36" s="7" t="n"/>
+      <c r="W36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -2129,15 +2150,15 @@
       <c r="H37" s="7" t="n"/>
       <c r="I37" s="7" t="n"/>
       <c r="J37" s="7" t="n"/>
-      <c r="K37" s="7" t="n"/>
-      <c r="L37" s="7" t="n"/>
-      <c r="M37" s="7" t="n"/>
-      <c r="N37" s="7" t="n"/>
       <c r="O37" s="7" t="n"/>
       <c r="P37" s="7" t="n"/>
       <c r="Q37" s="7" t="n"/>
       <c r="R37" s="7" t="n"/>
       <c r="S37" s="7" t="n"/>
+      <c r="T37" s="7" t="n"/>
+      <c r="U37" s="7" t="n"/>
+      <c r="V37" s="7" t="n"/>
+      <c r="W37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
@@ -2150,15 +2171,15 @@
       <c r="H38" s="7" t="n"/>
       <c r="I38" s="7" t="n"/>
       <c r="J38" s="7" t="n"/>
-      <c r="K38" s="7" t="n"/>
-      <c r="L38" s="7" t="n"/>
-      <c r="M38" s="7" t="n"/>
-      <c r="N38" s="7" t="n"/>
       <c r="O38" s="7" t="n"/>
       <c r="P38" s="7" t="n"/>
       <c r="Q38" s="7" t="n"/>
       <c r="R38" s="7" t="n"/>
       <c r="S38" s="7" t="n"/>
+      <c r="T38" s="7" t="n"/>
+      <c r="U38" s="7" t="n"/>
+      <c r="V38" s="7" t="n"/>
+      <c r="W38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n"/>
@@ -2171,15 +2192,15 @@
       <c r="H39" s="7" t="n"/>
       <c r="I39" s="7" t="n"/>
       <c r="J39" s="7" t="n"/>
-      <c r="K39" s="7" t="n"/>
-      <c r="L39" s="7" t="n"/>
-      <c r="M39" s="7" t="n"/>
-      <c r="N39" s="7" t="n"/>
       <c r="O39" s="7" t="n"/>
       <c r="P39" s="7" t="n"/>
       <c r="Q39" s="7" t="n"/>
       <c r="R39" s="7" t="n"/>
       <c r="S39" s="7" t="n"/>
+      <c r="T39" s="7" t="n"/>
+      <c r="U39" s="7" t="n"/>
+      <c r="V39" s="7" t="n"/>
+      <c r="W39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n"/>
@@ -2192,15 +2213,15 @@
       <c r="H40" s="7" t="n"/>
       <c r="I40" s="7" t="n"/>
       <c r="J40" s="7" t="n"/>
-      <c r="K40" s="7" t="n"/>
-      <c r="L40" s="7" t="n"/>
-      <c r="M40" s="7" t="n"/>
-      <c r="N40" s="7" t="n"/>
       <c r="O40" s="7" t="n"/>
       <c r="P40" s="7" t="n"/>
       <c r="Q40" s="7" t="n"/>
       <c r="R40" s="7" t="n"/>
       <c r="S40" s="7" t="n"/>
+      <c r="T40" s="7" t="n"/>
+      <c r="U40" s="7" t="n"/>
+      <c r="V40" s="7" t="n"/>
+      <c r="W40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n"/>
@@ -2213,15 +2234,15 @@
       <c r="H41" s="7" t="n"/>
       <c r="I41" s="7" t="n"/>
       <c r="J41" s="7" t="n"/>
-      <c r="K41" s="7" t="n"/>
-      <c r="L41" s="7" t="n"/>
-      <c r="M41" s="7" t="n"/>
-      <c r="N41" s="7" t="n"/>
       <c r="O41" s="7" t="n"/>
       <c r="P41" s="7" t="n"/>
       <c r="Q41" s="7" t="n"/>
       <c r="R41" s="7" t="n"/>
       <c r="S41" s="7" t="n"/>
+      <c r="T41" s="7" t="n"/>
+      <c r="U41" s="7" t="n"/>
+      <c r="V41" s="7" t="n"/>
+      <c r="W41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n"/>
@@ -2234,15 +2255,15 @@
       <c r="H42" s="7" t="n"/>
       <c r="I42" s="7" t="n"/>
       <c r="J42" s="7" t="n"/>
-      <c r="K42" s="7" t="n"/>
-      <c r="L42" s="7" t="n"/>
-      <c r="M42" s="7" t="n"/>
-      <c r="N42" s="7" t="n"/>
       <c r="O42" s="7" t="n"/>
       <c r="P42" s="7" t="n"/>
       <c r="Q42" s="7" t="n"/>
       <c r="R42" s="7" t="n"/>
       <c r="S42" s="7" t="n"/>
+      <c r="T42" s="7" t="n"/>
+      <c r="U42" s="7" t="n"/>
+      <c r="V42" s="7" t="n"/>
+      <c r="W42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n"/>
@@ -2255,15 +2276,15 @@
       <c r="H43" s="7" t="n"/>
       <c r="I43" s="7" t="n"/>
       <c r="J43" s="7" t="n"/>
-      <c r="K43" s="7" t="n"/>
-      <c r="L43" s="7" t="n"/>
-      <c r="M43" s="7" t="n"/>
-      <c r="N43" s="7" t="n"/>
       <c r="O43" s="7" t="n"/>
       <c r="P43" s="7" t="n"/>
       <c r="Q43" s="7" t="n"/>
       <c r="R43" s="7" t="n"/>
       <c r="S43" s="7" t="n"/>
+      <c r="T43" s="7" t="n"/>
+      <c r="U43" s="7" t="n"/>
+      <c r="V43" s="7" t="n"/>
+      <c r="W43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n"/>
@@ -2276,15 +2297,15 @@
       <c r="H44" s="7" t="n"/>
       <c r="I44" s="7" t="n"/>
       <c r="J44" s="7" t="n"/>
-      <c r="K44" s="7" t="n"/>
-      <c r="L44" s="7" t="n"/>
-      <c r="M44" s="7" t="n"/>
-      <c r="N44" s="7" t="n"/>
       <c r="O44" s="7" t="n"/>
       <c r="P44" s="7" t="n"/>
       <c r="Q44" s="7" t="n"/>
       <c r="R44" s="7" t="n"/>
       <c r="S44" s="7" t="n"/>
+      <c r="T44" s="7" t="n"/>
+      <c r="U44" s="7" t="n"/>
+      <c r="V44" s="7" t="n"/>
+      <c r="W44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n"/>
@@ -2297,15 +2318,15 @@
       <c r="H45" s="7" t="n"/>
       <c r="I45" s="7" t="n"/>
       <c r="J45" s="7" t="n"/>
-      <c r="K45" s="7" t="n"/>
-      <c r="L45" s="7" t="n"/>
-      <c r="M45" s="7" t="n"/>
-      <c r="N45" s="7" t="n"/>
       <c r="O45" s="7" t="n"/>
       <c r="P45" s="7" t="n"/>
       <c r="Q45" s="7" t="n"/>
       <c r="R45" s="7" t="n"/>
       <c r="S45" s="7" t="n"/>
+      <c r="T45" s="7" t="n"/>
+      <c r="U45" s="7" t="n"/>
+      <c r="V45" s="7" t="n"/>
+      <c r="W45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n"/>
@@ -2318,15 +2339,15 @@
       <c r="H46" s="7" t="n"/>
       <c r="I46" s="7" t="n"/>
       <c r="J46" s="7" t="n"/>
-      <c r="K46" s="7" t="n"/>
-      <c r="L46" s="7" t="n"/>
-      <c r="M46" s="7" t="n"/>
-      <c r="N46" s="7" t="n"/>
       <c r="O46" s="7" t="n"/>
       <c r="P46" s="7" t="n"/>
       <c r="Q46" s="7" t="n"/>
       <c r="R46" s="7" t="n"/>
       <c r="S46" s="7" t="n"/>
+      <c r="T46" s="7" t="n"/>
+      <c r="U46" s="7" t="n"/>
+      <c r="V46" s="7" t="n"/>
+      <c r="W46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n"/>
@@ -2339,15 +2360,15 @@
       <c r="H47" s="7" t="n"/>
       <c r="I47" s="7" t="n"/>
       <c r="J47" s="7" t="n"/>
-      <c r="K47" s="7" t="n"/>
-      <c r="L47" s="7" t="n"/>
-      <c r="M47" s="7" t="n"/>
-      <c r="N47" s="7" t="n"/>
       <c r="O47" s="7" t="n"/>
       <c r="P47" s="7" t="n"/>
       <c r="Q47" s="7" t="n"/>
       <c r="R47" s="7" t="n"/>
       <c r="S47" s="7" t="n"/>
+      <c r="T47" s="7" t="n"/>
+      <c r="U47" s="7" t="n"/>
+      <c r="V47" s="7" t="n"/>
+      <c r="W47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n"/>
@@ -2360,15 +2381,15 @@
       <c r="H48" s="7" t="n"/>
       <c r="I48" s="7" t="n"/>
       <c r="J48" s="7" t="n"/>
-      <c r="K48" s="7" t="n"/>
-      <c r="L48" s="7" t="n"/>
-      <c r="M48" s="7" t="n"/>
-      <c r="N48" s="7" t="n"/>
       <c r="O48" s="7" t="n"/>
       <c r="P48" s="7" t="n"/>
       <c r="Q48" s="7" t="n"/>
       <c r="R48" s="7" t="n"/>
       <c r="S48" s="7" t="n"/>
+      <c r="T48" s="7" t="n"/>
+      <c r="U48" s="7" t="n"/>
+      <c r="V48" s="7" t="n"/>
+      <c r="W48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n"/>
@@ -2381,15 +2402,15 @@
       <c r="H49" s="7" t="n"/>
       <c r="I49" s="7" t="n"/>
       <c r="J49" s="7" t="n"/>
-      <c r="K49" s="7" t="n"/>
-      <c r="L49" s="7" t="n"/>
-      <c r="M49" s="7" t="n"/>
-      <c r="N49" s="7" t="n"/>
       <c r="O49" s="7" t="n"/>
       <c r="P49" s="7" t="n"/>
       <c r="Q49" s="7" t="n"/>
       <c r="R49" s="7" t="n"/>
       <c r="S49" s="7" t="n"/>
+      <c r="T49" s="7" t="n"/>
+      <c r="U49" s="7" t="n"/>
+      <c r="V49" s="7" t="n"/>
+      <c r="W49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n"/>
@@ -2402,15 +2423,15 @@
       <c r="H50" s="7" t="n"/>
       <c r="I50" s="7" t="n"/>
       <c r="J50" s="7" t="n"/>
-      <c r="K50" s="7" t="n"/>
-      <c r="L50" s="7" t="n"/>
-      <c r="M50" s="7" t="n"/>
-      <c r="N50" s="7" t="n"/>
       <c r="O50" s="7" t="n"/>
       <c r="P50" s="7" t="n"/>
       <c r="Q50" s="7" t="n"/>
       <c r="R50" s="7" t="n"/>
       <c r="S50" s="7" t="n"/>
+      <c r="T50" s="7" t="n"/>
+      <c r="U50" s="7" t="n"/>
+      <c r="V50" s="7" t="n"/>
+      <c r="W50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="n"/>
@@ -2423,15 +2444,15 @@
       <c r="H51" s="7" t="n"/>
       <c r="I51" s="7" t="n"/>
       <c r="J51" s="7" t="n"/>
-      <c r="K51" s="7" t="n"/>
-      <c r="L51" s="7" t="n"/>
-      <c r="M51" s="7" t="n"/>
-      <c r="N51" s="7" t="n"/>
       <c r="O51" s="7" t="n"/>
       <c r="P51" s="7" t="n"/>
       <c r="Q51" s="7" t="n"/>
       <c r="R51" s="7" t="n"/>
       <c r="S51" s="7" t="n"/>
+      <c r="T51" s="7" t="n"/>
+      <c r="U51" s="7" t="n"/>
+      <c r="V51" s="7" t="n"/>
+      <c r="W51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n"/>
@@ -2444,15 +2465,15 @@
       <c r="H52" s="7" t="n"/>
       <c r="I52" s="7" t="n"/>
       <c r="J52" s="7" t="n"/>
-      <c r="K52" s="7" t="n"/>
-      <c r="L52" s="7" t="n"/>
-      <c r="M52" s="7" t="n"/>
-      <c r="N52" s="7" t="n"/>
       <c r="O52" s="7" t="n"/>
       <c r="P52" s="7" t="n"/>
       <c r="Q52" s="7" t="n"/>
       <c r="R52" s="7" t="n"/>
       <c r="S52" s="7" t="n"/>
+      <c r="T52" s="7" t="n"/>
+      <c r="U52" s="7" t="n"/>
+      <c r="V52" s="7" t="n"/>
+      <c r="W52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="n"/>
@@ -2465,15 +2486,15 @@
       <c r="H53" s="7" t="n"/>
       <c r="I53" s="7" t="n"/>
       <c r="J53" s="7" t="n"/>
-      <c r="K53" s="7" t="n"/>
-      <c r="L53" s="7" t="n"/>
-      <c r="M53" s="7" t="n"/>
-      <c r="N53" s="7" t="n"/>
       <c r="O53" s="7" t="n"/>
       <c r="P53" s="7" t="n"/>
       <c r="Q53" s="7" t="n"/>
       <c r="R53" s="7" t="n"/>
       <c r="S53" s="7" t="n"/>
+      <c r="T53" s="7" t="n"/>
+      <c r="U53" s="7" t="n"/>
+      <c r="V53" s="7" t="n"/>
+      <c r="W53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n"/>
@@ -2486,15 +2507,15 @@
       <c r="H54" s="7" t="n"/>
       <c r="I54" s="7" t="n"/>
       <c r="J54" s="7" t="n"/>
-      <c r="K54" s="7" t="n"/>
-      <c r="L54" s="7" t="n"/>
-      <c r="M54" s="7" t="n"/>
-      <c r="N54" s="7" t="n"/>
       <c r="O54" s="7" t="n"/>
       <c r="P54" s="7" t="n"/>
       <c r="Q54" s="7" t="n"/>
       <c r="R54" s="7" t="n"/>
       <c r="S54" s="7" t="n"/>
+      <c r="T54" s="7" t="n"/>
+      <c r="U54" s="7" t="n"/>
+      <c r="V54" s="7" t="n"/>
+      <c r="W54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n"/>
@@ -2507,15 +2528,15 @@
       <c r="H55" s="7" t="n"/>
       <c r="I55" s="7" t="n"/>
       <c r="J55" s="7" t="n"/>
-      <c r="K55" s="7" t="n"/>
-      <c r="L55" s="7" t="n"/>
-      <c r="M55" s="7" t="n"/>
-      <c r="N55" s="7" t="n"/>
       <c r="O55" s="7" t="n"/>
       <c r="P55" s="7" t="n"/>
       <c r="Q55" s="7" t="n"/>
       <c r="R55" s="7" t="n"/>
       <c r="S55" s="7" t="n"/>
+      <c r="T55" s="7" t="n"/>
+      <c r="U55" s="7" t="n"/>
+      <c r="V55" s="7" t="n"/>
+      <c r="W55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n"/>
@@ -2528,15 +2549,15 @@
       <c r="H56" s="7" t="n"/>
       <c r="I56" s="7" t="n"/>
       <c r="J56" s="7" t="n"/>
-      <c r="K56" s="7" t="n"/>
-      <c r="L56" s="7" t="n"/>
-      <c r="M56" s="7" t="n"/>
-      <c r="N56" s="7" t="n"/>
       <c r="O56" s="7" t="n"/>
       <c r="P56" s="7" t="n"/>
       <c r="Q56" s="7" t="n"/>
       <c r="R56" s="7" t="n"/>
       <c r="S56" s="7" t="n"/>
+      <c r="T56" s="7" t="n"/>
+      <c r="U56" s="7" t="n"/>
+      <c r="V56" s="7" t="n"/>
+      <c r="W56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n"/>
@@ -2549,15 +2570,15 @@
       <c r="H57" s="7" t="n"/>
       <c r="I57" s="7" t="n"/>
       <c r="J57" s="7" t="n"/>
-      <c r="K57" s="7" t="n"/>
-      <c r="L57" s="7" t="n"/>
-      <c r="M57" s="7" t="n"/>
-      <c r="N57" s="7" t="n"/>
       <c r="O57" s="7" t="n"/>
       <c r="P57" s="7" t="n"/>
       <c r="Q57" s="7" t="n"/>
       <c r="R57" s="7" t="n"/>
       <c r="S57" s="7" t="n"/>
+      <c r="T57" s="7" t="n"/>
+      <c r="U57" s="7" t="n"/>
+      <c r="V57" s="7" t="n"/>
+      <c r="W57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n"/>
@@ -2570,15 +2591,15 @@
       <c r="H58" s="7" t="n"/>
       <c r="I58" s="7" t="n"/>
       <c r="J58" s="7" t="n"/>
-      <c r="K58" s="7" t="n"/>
-      <c r="L58" s="7" t="n"/>
-      <c r="M58" s="7" t="n"/>
-      <c r="N58" s="7" t="n"/>
       <c r="O58" s="7" t="n"/>
       <c r="P58" s="7" t="n"/>
       <c r="Q58" s="7" t="n"/>
       <c r="R58" s="7" t="n"/>
       <c r="S58" s="7" t="n"/>
+      <c r="T58" s="7" t="n"/>
+      <c r="U58" s="7" t="n"/>
+      <c r="V58" s="7" t="n"/>
+      <c r="W58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n"/>
@@ -2591,15 +2612,15 @@
       <c r="H59" s="7" t="n"/>
       <c r="I59" s="7" t="n"/>
       <c r="J59" s="7" t="n"/>
-      <c r="K59" s="7" t="n"/>
-      <c r="L59" s="7" t="n"/>
-      <c r="M59" s="7" t="n"/>
-      <c r="N59" s="7" t="n"/>
       <c r="O59" s="7" t="n"/>
       <c r="P59" s="7" t="n"/>
       <c r="Q59" s="7" t="n"/>
       <c r="R59" s="7" t="n"/>
       <c r="S59" s="7" t="n"/>
+      <c r="T59" s="7" t="n"/>
+      <c r="U59" s="7" t="n"/>
+      <c r="V59" s="7" t="n"/>
+      <c r="W59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n"/>
@@ -2612,15 +2633,15 @@
       <c r="H60" s="7" t="n"/>
       <c r="I60" s="7" t="n"/>
       <c r="J60" s="7" t="n"/>
-      <c r="K60" s="7" t="n"/>
-      <c r="L60" s="7" t="n"/>
-      <c r="M60" s="7" t="n"/>
-      <c r="N60" s="7" t="n"/>
       <c r="O60" s="7" t="n"/>
       <c r="P60" s="7" t="n"/>
       <c r="Q60" s="7" t="n"/>
       <c r="R60" s="7" t="n"/>
       <c r="S60" s="7" t="n"/>
+      <c r="T60" s="7" t="n"/>
+      <c r="U60" s="7" t="n"/>
+      <c r="V60" s="7" t="n"/>
+      <c r="W60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="n"/>
@@ -2633,15 +2654,15 @@
       <c r="H61" s="7" t="n"/>
       <c r="I61" s="7" t="n"/>
       <c r="J61" s="7" t="n"/>
-      <c r="K61" s="7" t="n"/>
-      <c r="L61" s="7" t="n"/>
-      <c r="M61" s="7" t="n"/>
-      <c r="N61" s="7" t="n"/>
       <c r="O61" s="7" t="n"/>
       <c r="P61" s="7" t="n"/>
       <c r="Q61" s="7" t="n"/>
       <c r="R61" s="7" t="n"/>
       <c r="S61" s="7" t="n"/>
+      <c r="T61" s="7" t="n"/>
+      <c r="U61" s="7" t="n"/>
+      <c r="V61" s="7" t="n"/>
+      <c r="W61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n"/>
@@ -2654,15 +2675,15 @@
       <c r="H62" s="7" t="n"/>
       <c r="I62" s="7" t="n"/>
       <c r="J62" s="7" t="n"/>
-      <c r="K62" s="7" t="n"/>
-      <c r="L62" s="7" t="n"/>
-      <c r="M62" s="7" t="n"/>
-      <c r="N62" s="7" t="n"/>
       <c r="O62" s="7" t="n"/>
       <c r="P62" s="7" t="n"/>
       <c r="Q62" s="7" t="n"/>
       <c r="R62" s="7" t="n"/>
       <c r="S62" s="7" t="n"/>
+      <c r="T62" s="7" t="n"/>
+      <c r="U62" s="7" t="n"/>
+      <c r="V62" s="7" t="n"/>
+      <c r="W62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="n"/>
@@ -2675,15 +2696,15 @@
       <c r="H63" s="7" t="n"/>
       <c r="I63" s="7" t="n"/>
       <c r="J63" s="7" t="n"/>
-      <c r="K63" s="7" t="n"/>
-      <c r="L63" s="7" t="n"/>
-      <c r="M63" s="7" t="n"/>
-      <c r="N63" s="7" t="n"/>
       <c r="O63" s="7" t="n"/>
       <c r="P63" s="7" t="n"/>
       <c r="Q63" s="7" t="n"/>
       <c r="R63" s="7" t="n"/>
       <c r="S63" s="7" t="n"/>
+      <c r="T63" s="7" t="n"/>
+      <c r="U63" s="7" t="n"/>
+      <c r="V63" s="7" t="n"/>
+      <c r="W63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n"/>
@@ -2696,15 +2717,15 @@
       <c r="H64" s="7" t="n"/>
       <c r="I64" s="7" t="n"/>
       <c r="J64" s="7" t="n"/>
-      <c r="K64" s="7" t="n"/>
-      <c r="L64" s="7" t="n"/>
-      <c r="M64" s="7" t="n"/>
-      <c r="N64" s="7" t="n"/>
       <c r="O64" s="7" t="n"/>
       <c r="P64" s="7" t="n"/>
       <c r="Q64" s="7" t="n"/>
       <c r="R64" s="7" t="n"/>
       <c r="S64" s="7" t="n"/>
+      <c r="T64" s="7" t="n"/>
+      <c r="U64" s="7" t="n"/>
+      <c r="V64" s="7" t="n"/>
+      <c r="W64" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="n"/>
@@ -2717,15 +2738,15 @@
       <c r="H65" s="7" t="n"/>
       <c r="I65" s="7" t="n"/>
       <c r="J65" s="7" t="n"/>
-      <c r="K65" s="7" t="n"/>
-      <c r="L65" s="7" t="n"/>
-      <c r="M65" s="7" t="n"/>
-      <c r="N65" s="7" t="n"/>
       <c r="O65" s="7" t="n"/>
       <c r="P65" s="7" t="n"/>
       <c r="Q65" s="7" t="n"/>
       <c r="R65" s="7" t="n"/>
       <c r="S65" s="7" t="n"/>
+      <c r="T65" s="7" t="n"/>
+      <c r="U65" s="7" t="n"/>
+      <c r="V65" s="7" t="n"/>
+      <c r="W65" s="7" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n"/>
@@ -2738,15 +2759,15 @@
       <c r="H66" s="7" t="n"/>
       <c r="I66" s="7" t="n"/>
       <c r="J66" s="7" t="n"/>
-      <c r="K66" s="7" t="n"/>
-      <c r="L66" s="7" t="n"/>
-      <c r="M66" s="7" t="n"/>
-      <c r="N66" s="7" t="n"/>
       <c r="O66" s="7" t="n"/>
       <c r="P66" s="7" t="n"/>
       <c r="Q66" s="7" t="n"/>
       <c r="R66" s="7" t="n"/>
       <c r="S66" s="7" t="n"/>
+      <c r="T66" s="7" t="n"/>
+      <c r="U66" s="7" t="n"/>
+      <c r="V66" s="7" t="n"/>
+      <c r="W66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="n"/>
@@ -2759,15 +2780,15 @@
       <c r="H67" s="7" t="n"/>
       <c r="I67" s="7" t="n"/>
       <c r="J67" s="7" t="n"/>
-      <c r="K67" s="7" t="n"/>
-      <c r="L67" s="7" t="n"/>
-      <c r="M67" s="7" t="n"/>
-      <c r="N67" s="7" t="n"/>
       <c r="O67" s="7" t="n"/>
       <c r="P67" s="7" t="n"/>
       <c r="Q67" s="7" t="n"/>
       <c r="R67" s="7" t="n"/>
       <c r="S67" s="7" t="n"/>
+      <c r="T67" s="7" t="n"/>
+      <c r="U67" s="7" t="n"/>
+      <c r="V67" s="7" t="n"/>
+      <c r="W67" s="7" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="n"/>
@@ -2780,15 +2801,15 @@
       <c r="H68" s="7" t="n"/>
       <c r="I68" s="7" t="n"/>
       <c r="J68" s="7" t="n"/>
-      <c r="K68" s="7" t="n"/>
-      <c r="L68" s="7" t="n"/>
-      <c r="M68" s="7" t="n"/>
-      <c r="N68" s="7" t="n"/>
       <c r="O68" s="7" t="n"/>
       <c r="P68" s="7" t="n"/>
       <c r="Q68" s="7" t="n"/>
       <c r="R68" s="7" t="n"/>
       <c r="S68" s="7" t="n"/>
+      <c r="T68" s="7" t="n"/>
+      <c r="U68" s="7" t="n"/>
+      <c r="V68" s="7" t="n"/>
+      <c r="W68" s="7" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="n"/>
@@ -2801,15 +2822,15 @@
       <c r="H69" s="7" t="n"/>
       <c r="I69" s="7" t="n"/>
       <c r="J69" s="7" t="n"/>
-      <c r="K69" s="7" t="n"/>
-      <c r="L69" s="7" t="n"/>
-      <c r="M69" s="7" t="n"/>
-      <c r="N69" s="7" t="n"/>
       <c r="O69" s="7" t="n"/>
       <c r="P69" s="7" t="n"/>
       <c r="Q69" s="7" t="n"/>
       <c r="R69" s="7" t="n"/>
       <c r="S69" s="7" t="n"/>
+      <c r="T69" s="7" t="n"/>
+      <c r="U69" s="7" t="n"/>
+      <c r="V69" s="7" t="n"/>
+      <c r="W69" s="7" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="n"/>
@@ -2822,15 +2843,15 @@
       <c r="H70" s="7" t="n"/>
       <c r="I70" s="7" t="n"/>
       <c r="J70" s="7" t="n"/>
-      <c r="K70" s="7" t="n"/>
-      <c r="L70" s="7" t="n"/>
-      <c r="M70" s="7" t="n"/>
-      <c r="N70" s="7" t="n"/>
       <c r="O70" s="7" t="n"/>
       <c r="P70" s="7" t="n"/>
       <c r="Q70" s="7" t="n"/>
       <c r="R70" s="7" t="n"/>
       <c r="S70" s="7" t="n"/>
+      <c r="T70" s="7" t="n"/>
+      <c r="U70" s="7" t="n"/>
+      <c r="V70" s="7" t="n"/>
+      <c r="W70" s="7" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="n"/>
@@ -2843,15 +2864,15 @@
       <c r="H71" s="7" t="n"/>
       <c r="I71" s="7" t="n"/>
       <c r="J71" s="7" t="n"/>
-      <c r="K71" s="7" t="n"/>
-      <c r="L71" s="7" t="n"/>
-      <c r="M71" s="7" t="n"/>
-      <c r="N71" s="7" t="n"/>
       <c r="O71" s="7" t="n"/>
       <c r="P71" s="7" t="n"/>
       <c r="Q71" s="7" t="n"/>
       <c r="R71" s="7" t="n"/>
       <c r="S71" s="7" t="n"/>
+      <c r="T71" s="7" t="n"/>
+      <c r="U71" s="7" t="n"/>
+      <c r="V71" s="7" t="n"/>
+      <c r="W71" s="7" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n"/>
@@ -2864,15 +2885,15 @@
       <c r="H72" s="7" t="n"/>
       <c r="I72" s="7" t="n"/>
       <c r="J72" s="7" t="n"/>
-      <c r="K72" s="7" t="n"/>
-      <c r="L72" s="7" t="n"/>
-      <c r="M72" s="7" t="n"/>
-      <c r="N72" s="7" t="n"/>
       <c r="O72" s="7" t="n"/>
       <c r="P72" s="7" t="n"/>
       <c r="Q72" s="7" t="n"/>
       <c r="R72" s="7" t="n"/>
       <c r="S72" s="7" t="n"/>
+      <c r="T72" s="7" t="n"/>
+      <c r="U72" s="7" t="n"/>
+      <c r="V72" s="7" t="n"/>
+      <c r="W72" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="n"/>
@@ -2885,15 +2906,15 @@
       <c r="H73" s="7" t="n"/>
       <c r="I73" s="7" t="n"/>
       <c r="J73" s="7" t="n"/>
-      <c r="K73" s="7" t="n"/>
-      <c r="L73" s="7" t="n"/>
-      <c r="M73" s="7" t="n"/>
-      <c r="N73" s="7" t="n"/>
       <c r="O73" s="7" t="n"/>
       <c r="P73" s="7" t="n"/>
       <c r="Q73" s="7" t="n"/>
       <c r="R73" s="7" t="n"/>
       <c r="S73" s="7" t="n"/>
+      <c r="T73" s="7" t="n"/>
+      <c r="U73" s="7" t="n"/>
+      <c r="V73" s="7" t="n"/>
+      <c r="W73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="n"/>
@@ -2906,15 +2927,15 @@
       <c r="H74" s="7" t="n"/>
       <c r="I74" s="7" t="n"/>
       <c r="J74" s="7" t="n"/>
-      <c r="K74" s="7" t="n"/>
-      <c r="L74" s="7" t="n"/>
-      <c r="M74" s="7" t="n"/>
-      <c r="N74" s="7" t="n"/>
       <c r="O74" s="7" t="n"/>
       <c r="P74" s="7" t="n"/>
       <c r="Q74" s="7" t="n"/>
       <c r="R74" s="7" t="n"/>
       <c r="S74" s="7" t="n"/>
+      <c r="T74" s="7" t="n"/>
+      <c r="U74" s="7" t="n"/>
+      <c r="V74" s="7" t="n"/>
+      <c r="W74" s="7" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="n"/>
@@ -2927,15 +2948,15 @@
       <c r="H75" s="7" t="n"/>
       <c r="I75" s="7" t="n"/>
       <c r="J75" s="7" t="n"/>
-      <c r="K75" s="7" t="n"/>
-      <c r="L75" s="7" t="n"/>
-      <c r="M75" s="7" t="n"/>
-      <c r="N75" s="7" t="n"/>
       <c r="O75" s="7" t="n"/>
       <c r="P75" s="7" t="n"/>
       <c r="Q75" s="7" t="n"/>
       <c r="R75" s="7" t="n"/>
       <c r="S75" s="7" t="n"/>
+      <c r="T75" s="7" t="n"/>
+      <c r="U75" s="7" t="n"/>
+      <c r="V75" s="7" t="n"/>
+      <c r="W75" s="7" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="n"/>
@@ -2948,15 +2969,15 @@
       <c r="H76" s="7" t="n"/>
       <c r="I76" s="7" t="n"/>
       <c r="J76" s="7" t="n"/>
-      <c r="K76" s="7" t="n"/>
-      <c r="L76" s="7" t="n"/>
-      <c r="M76" s="7" t="n"/>
-      <c r="N76" s="7" t="n"/>
       <c r="O76" s="7" t="n"/>
       <c r="P76" s="7" t="n"/>
       <c r="Q76" s="7" t="n"/>
       <c r="R76" s="7" t="n"/>
       <c r="S76" s="7" t="n"/>
+      <c r="T76" s="7" t="n"/>
+      <c r="U76" s="7" t="n"/>
+      <c r="V76" s="7" t="n"/>
+      <c r="W76" s="7" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="n"/>
@@ -2969,15 +2990,15 @@
       <c r="H77" s="7" t="n"/>
       <c r="I77" s="7" t="n"/>
       <c r="J77" s="7" t="n"/>
-      <c r="K77" s="7" t="n"/>
-      <c r="L77" s="7" t="n"/>
-      <c r="M77" s="7" t="n"/>
-      <c r="N77" s="7" t="n"/>
       <c r="O77" s="7" t="n"/>
       <c r="P77" s="7" t="n"/>
       <c r="Q77" s="7" t="n"/>
       <c r="R77" s="7" t="n"/>
       <c r="S77" s="7" t="n"/>
+      <c r="T77" s="7" t="n"/>
+      <c r="U77" s="7" t="n"/>
+      <c r="V77" s="7" t="n"/>
+      <c r="W77" s="7" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="n"/>
@@ -2990,15 +3011,15 @@
       <c r="H78" s="7" t="n"/>
       <c r="I78" s="7" t="n"/>
       <c r="J78" s="7" t="n"/>
-      <c r="K78" s="7" t="n"/>
-      <c r="L78" s="7" t="n"/>
-      <c r="M78" s="7" t="n"/>
-      <c r="N78" s="7" t="n"/>
       <c r="O78" s="7" t="n"/>
       <c r="P78" s="7" t="n"/>
       <c r="Q78" s="7" t="n"/>
       <c r="R78" s="7" t="n"/>
       <c r="S78" s="7" t="n"/>
+      <c r="T78" s="7" t="n"/>
+      <c r="U78" s="7" t="n"/>
+      <c r="V78" s="7" t="n"/>
+      <c r="W78" s="7" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="n"/>
@@ -3011,15 +3032,15 @@
       <c r="H79" s="7" t="n"/>
       <c r="I79" s="7" t="n"/>
       <c r="J79" s="7" t="n"/>
-      <c r="K79" s="7" t="n"/>
-      <c r="L79" s="7" t="n"/>
-      <c r="M79" s="7" t="n"/>
-      <c r="N79" s="7" t="n"/>
       <c r="O79" s="7" t="n"/>
       <c r="P79" s="7" t="n"/>
       <c r="Q79" s="7" t="n"/>
       <c r="R79" s="7" t="n"/>
       <c r="S79" s="7" t="n"/>
+      <c r="T79" s="7" t="n"/>
+      <c r="U79" s="7" t="n"/>
+      <c r="V79" s="7" t="n"/>
+      <c r="W79" s="7" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="n"/>
@@ -3032,15 +3053,15 @@
       <c r="H80" s="7" t="n"/>
       <c r="I80" s="7" t="n"/>
       <c r="J80" s="7" t="n"/>
-      <c r="K80" s="7" t="n"/>
-      <c r="L80" s="7" t="n"/>
-      <c r="M80" s="7" t="n"/>
-      <c r="N80" s="7" t="n"/>
       <c r="O80" s="7" t="n"/>
       <c r="P80" s="7" t="n"/>
       <c r="Q80" s="7" t="n"/>
       <c r="R80" s="7" t="n"/>
       <c r="S80" s="7" t="n"/>
+      <c r="T80" s="7" t="n"/>
+      <c r="U80" s="7" t="n"/>
+      <c r="V80" s="7" t="n"/>
+      <c r="W80" s="7" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="n"/>
@@ -3053,15 +3074,15 @@
       <c r="H81" s="7" t="n"/>
       <c r="I81" s="7" t="n"/>
       <c r="J81" s="7" t="n"/>
-      <c r="K81" s="7" t="n"/>
-      <c r="L81" s="7" t="n"/>
-      <c r="M81" s="7" t="n"/>
-      <c r="N81" s="7" t="n"/>
       <c r="O81" s="7" t="n"/>
       <c r="P81" s="7" t="n"/>
       <c r="Q81" s="7" t="n"/>
       <c r="R81" s="7" t="n"/>
       <c r="S81" s="7" t="n"/>
+      <c r="T81" s="7" t="n"/>
+      <c r="U81" s="7" t="n"/>
+      <c r="V81" s="7" t="n"/>
+      <c r="W81" s="7" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="n"/>
@@ -3074,15 +3095,15 @@
       <c r="H82" s="7" t="n"/>
       <c r="I82" s="7" t="n"/>
       <c r="J82" s="7" t="n"/>
-      <c r="K82" s="7" t="n"/>
-      <c r="L82" s="7" t="n"/>
-      <c r="M82" s="7" t="n"/>
-      <c r="N82" s="7" t="n"/>
       <c r="O82" s="7" t="n"/>
       <c r="P82" s="7" t="n"/>
       <c r="Q82" s="7" t="n"/>
       <c r="R82" s="7" t="n"/>
       <c r="S82" s="7" t="n"/>
+      <c r="T82" s="7" t="n"/>
+      <c r="U82" s="7" t="n"/>
+      <c r="V82" s="7" t="n"/>
+      <c r="W82" s="7" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="n"/>
@@ -3095,15 +3116,15 @@
       <c r="H83" s="7" t="n"/>
       <c r="I83" s="7" t="n"/>
       <c r="J83" s="7" t="n"/>
-      <c r="K83" s="7" t="n"/>
-      <c r="L83" s="7" t="n"/>
-      <c r="M83" s="7" t="n"/>
-      <c r="N83" s="7" t="n"/>
       <c r="O83" s="7" t="n"/>
       <c r="P83" s="7" t="n"/>
       <c r="Q83" s="7" t="n"/>
       <c r="R83" s="7" t="n"/>
       <c r="S83" s="7" t="n"/>
+      <c r="T83" s="7" t="n"/>
+      <c r="U83" s="7" t="n"/>
+      <c r="V83" s="7" t="n"/>
+      <c r="W83" s="7" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="n"/>
@@ -3116,15 +3137,15 @@
       <c r="H84" s="7" t="n"/>
       <c r="I84" s="7" t="n"/>
       <c r="J84" s="7" t="n"/>
-      <c r="K84" s="7" t="n"/>
-      <c r="L84" s="7" t="n"/>
-      <c r="M84" s="7" t="n"/>
-      <c r="N84" s="7" t="n"/>
       <c r="O84" s="7" t="n"/>
       <c r="P84" s="7" t="n"/>
       <c r="Q84" s="7" t="n"/>
       <c r="R84" s="7" t="n"/>
       <c r="S84" s="7" t="n"/>
+      <c r="T84" s="7" t="n"/>
+      <c r="U84" s="7" t="n"/>
+      <c r="V84" s="7" t="n"/>
+      <c r="W84" s="7" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="n"/>
@@ -3137,15 +3158,15 @@
       <c r="H85" s="7" t="n"/>
       <c r="I85" s="7" t="n"/>
       <c r="J85" s="7" t="n"/>
-      <c r="K85" s="7" t="n"/>
-      <c r="L85" s="7" t="n"/>
-      <c r="M85" s="7" t="n"/>
-      <c r="N85" s="7" t="n"/>
       <c r="O85" s="7" t="n"/>
       <c r="P85" s="7" t="n"/>
       <c r="Q85" s="7" t="n"/>
       <c r="R85" s="7" t="n"/>
       <c r="S85" s="7" t="n"/>
+      <c r="T85" s="7" t="n"/>
+      <c r="U85" s="7" t="n"/>
+      <c r="V85" s="7" t="n"/>
+      <c r="W85" s="7" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="n"/>
@@ -3158,15 +3179,15 @@
       <c r="H86" s="7" t="n"/>
       <c r="I86" s="7" t="n"/>
       <c r="J86" s="7" t="n"/>
-      <c r="K86" s="7" t="n"/>
-      <c r="L86" s="7" t="n"/>
-      <c r="M86" s="7" t="n"/>
-      <c r="N86" s="7" t="n"/>
       <c r="O86" s="7" t="n"/>
       <c r="P86" s="7" t="n"/>
       <c r="Q86" s="7" t="n"/>
       <c r="R86" s="7" t="n"/>
       <c r="S86" s="7" t="n"/>
+      <c r="T86" s="7" t="n"/>
+      <c r="U86" s="7" t="n"/>
+      <c r="V86" s="7" t="n"/>
+      <c r="W86" s="7" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="n"/>
@@ -3179,15 +3200,15 @@
       <c r="H87" s="7" t="n"/>
       <c r="I87" s="7" t="n"/>
       <c r="J87" s="7" t="n"/>
-      <c r="K87" s="7" t="n"/>
-      <c r="L87" s="7" t="n"/>
-      <c r="M87" s="7" t="n"/>
-      <c r="N87" s="7" t="n"/>
       <c r="O87" s="7" t="n"/>
       <c r="P87" s="7" t="n"/>
       <c r="Q87" s="7" t="n"/>
       <c r="R87" s="7" t="n"/>
       <c r="S87" s="7" t="n"/>
+      <c r="T87" s="7" t="n"/>
+      <c r="U87" s="7" t="n"/>
+      <c r="V87" s="7" t="n"/>
+      <c r="W87" s="7" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="n"/>
@@ -3200,15 +3221,15 @@
       <c r="H88" s="7" t="n"/>
       <c r="I88" s="7" t="n"/>
       <c r="J88" s="7" t="n"/>
-      <c r="K88" s="7" t="n"/>
-      <c r="L88" s="7" t="n"/>
-      <c r="M88" s="7" t="n"/>
-      <c r="N88" s="7" t="n"/>
       <c r="O88" s="7" t="n"/>
       <c r="P88" s="7" t="n"/>
       <c r="Q88" s="7" t="n"/>
       <c r="R88" s="7" t="n"/>
       <c r="S88" s="7" t="n"/>
+      <c r="T88" s="7" t="n"/>
+      <c r="U88" s="7" t="n"/>
+      <c r="V88" s="7" t="n"/>
+      <c r="W88" s="7" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="n"/>
@@ -3221,15 +3242,15 @@
       <c r="H89" s="7" t="n"/>
       <c r="I89" s="7" t="n"/>
       <c r="J89" s="7" t="n"/>
-      <c r="K89" s="7" t="n"/>
-      <c r="L89" s="7" t="n"/>
-      <c r="M89" s="7" t="n"/>
-      <c r="N89" s="7" t="n"/>
       <c r="O89" s="7" t="n"/>
       <c r="P89" s="7" t="n"/>
       <c r="Q89" s="7" t="n"/>
       <c r="R89" s="7" t="n"/>
       <c r="S89" s="7" t="n"/>
+      <c r="T89" s="7" t="n"/>
+      <c r="U89" s="7" t="n"/>
+      <c r="V89" s="7" t="n"/>
+      <c r="W89" s="7" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="n"/>
@@ -3242,15 +3263,15 @@
       <c r="H90" s="7" t="n"/>
       <c r="I90" s="7" t="n"/>
       <c r="J90" s="7" t="n"/>
-      <c r="K90" s="7" t="n"/>
-      <c r="L90" s="7" t="n"/>
-      <c r="M90" s="7" t="n"/>
-      <c r="N90" s="7" t="n"/>
       <c r="O90" s="7" t="n"/>
       <c r="P90" s="7" t="n"/>
       <c r="Q90" s="7" t="n"/>
       <c r="R90" s="7" t="n"/>
       <c r="S90" s="7" t="n"/>
+      <c r="T90" s="7" t="n"/>
+      <c r="U90" s="7" t="n"/>
+      <c r="V90" s="7" t="n"/>
+      <c r="W90" s="7" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="n"/>
@@ -3263,15 +3284,15 @@
       <c r="H91" s="7" t="n"/>
       <c r="I91" s="7" t="n"/>
       <c r="J91" s="7" t="n"/>
-      <c r="K91" s="7" t="n"/>
-      <c r="L91" s="7" t="n"/>
-      <c r="M91" s="7" t="n"/>
-      <c r="N91" s="7" t="n"/>
       <c r="O91" s="7" t="n"/>
       <c r="P91" s="7" t="n"/>
       <c r="Q91" s="7" t="n"/>
       <c r="R91" s="7" t="n"/>
       <c r="S91" s="7" t="n"/>
+      <c r="T91" s="7" t="n"/>
+      <c r="U91" s="7" t="n"/>
+      <c r="V91" s="7" t="n"/>
+      <c r="W91" s="7" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="n"/>
@@ -3284,15 +3305,15 @@
       <c r="H92" s="7" t="n"/>
       <c r="I92" s="7" t="n"/>
       <c r="J92" s="7" t="n"/>
-      <c r="K92" s="7" t="n"/>
-      <c r="L92" s="7" t="n"/>
-      <c r="M92" s="7" t="n"/>
-      <c r="N92" s="7" t="n"/>
       <c r="O92" s="7" t="n"/>
       <c r="P92" s="7" t="n"/>
       <c r="Q92" s="7" t="n"/>
       <c r="R92" s="7" t="n"/>
       <c r="S92" s="7" t="n"/>
+      <c r="T92" s="7" t="n"/>
+      <c r="U92" s="7" t="n"/>
+      <c r="V92" s="7" t="n"/>
+      <c r="W92" s="7" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="n"/>
@@ -3305,15 +3326,15 @@
       <c r="H93" s="7" t="n"/>
       <c r="I93" s="7" t="n"/>
       <c r="J93" s="7" t="n"/>
-      <c r="K93" s="7" t="n"/>
-      <c r="L93" s="7" t="n"/>
-      <c r="M93" s="7" t="n"/>
-      <c r="N93" s="7" t="n"/>
       <c r="O93" s="7" t="n"/>
       <c r="P93" s="7" t="n"/>
       <c r="Q93" s="7" t="n"/>
       <c r="R93" s="7" t="n"/>
       <c r="S93" s="7" t="n"/>
+      <c r="T93" s="7" t="n"/>
+      <c r="U93" s="7" t="n"/>
+      <c r="V93" s="7" t="n"/>
+      <c r="W93" s="7" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="n"/>
@@ -3326,15 +3347,15 @@
       <c r="H94" s="7" t="n"/>
       <c r="I94" s="7" t="n"/>
       <c r="J94" s="7" t="n"/>
-      <c r="K94" s="7" t="n"/>
-      <c r="L94" s="7" t="n"/>
-      <c r="M94" s="7" t="n"/>
-      <c r="N94" s="7" t="n"/>
       <c r="O94" s="7" t="n"/>
       <c r="P94" s="7" t="n"/>
       <c r="Q94" s="7" t="n"/>
       <c r="R94" s="7" t="n"/>
       <c r="S94" s="7" t="n"/>
+      <c r="T94" s="7" t="n"/>
+      <c r="U94" s="7" t="n"/>
+      <c r="V94" s="7" t="n"/>
+      <c r="W94" s="7" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="n"/>
@@ -3347,15 +3368,15 @@
       <c r="H95" s="7" t="n"/>
       <c r="I95" s="7" t="n"/>
       <c r="J95" s="7" t="n"/>
-      <c r="K95" s="7" t="n"/>
-      <c r="L95" s="7" t="n"/>
-      <c r="M95" s="7" t="n"/>
-      <c r="N95" s="7" t="n"/>
       <c r="O95" s="7" t="n"/>
       <c r="P95" s="7" t="n"/>
       <c r="Q95" s="7" t="n"/>
       <c r="R95" s="7" t="n"/>
       <c r="S95" s="7" t="n"/>
+      <c r="T95" s="7" t="n"/>
+      <c r="U95" s="7" t="n"/>
+      <c r="V95" s="7" t="n"/>
+      <c r="W95" s="7" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="n"/>
@@ -3368,15 +3389,15 @@
       <c r="H96" s="7" t="n"/>
       <c r="I96" s="7" t="n"/>
       <c r="J96" s="7" t="n"/>
-      <c r="K96" s="7" t="n"/>
-      <c r="L96" s="7" t="n"/>
-      <c r="M96" s="7" t="n"/>
-      <c r="N96" s="7" t="n"/>
       <c r="O96" s="7" t="n"/>
       <c r="P96" s="7" t="n"/>
       <c r="Q96" s="7" t="n"/>
       <c r="R96" s="7" t="n"/>
       <c r="S96" s="7" t="n"/>
+      <c r="T96" s="7" t="n"/>
+      <c r="U96" s="7" t="n"/>
+      <c r="V96" s="7" t="n"/>
+      <c r="W96" s="7" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="n"/>
@@ -3389,15 +3410,15 @@
       <c r="H97" s="7" t="n"/>
       <c r="I97" s="7" t="n"/>
       <c r="J97" s="7" t="n"/>
-      <c r="K97" s="7" t="n"/>
-      <c r="L97" s="7" t="n"/>
-      <c r="M97" s="7" t="n"/>
-      <c r="N97" s="7" t="n"/>
       <c r="O97" s="7" t="n"/>
       <c r="P97" s="7" t="n"/>
       <c r="Q97" s="7" t="n"/>
       <c r="R97" s="7" t="n"/>
       <c r="S97" s="7" t="n"/>
+      <c r="T97" s="7" t="n"/>
+      <c r="U97" s="7" t="n"/>
+      <c r="V97" s="7" t="n"/>
+      <c r="W97" s="7" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="n"/>
@@ -3410,15 +3431,15 @@
       <c r="H98" s="7" t="n"/>
       <c r="I98" s="7" t="n"/>
       <c r="J98" s="7" t="n"/>
-      <c r="K98" s="7" t="n"/>
-      <c r="L98" s="7" t="n"/>
-      <c r="M98" s="7" t="n"/>
-      <c r="N98" s="7" t="n"/>
       <c r="O98" s="7" t="n"/>
       <c r="P98" s="7" t="n"/>
       <c r="Q98" s="7" t="n"/>
       <c r="R98" s="7" t="n"/>
       <c r="S98" s="7" t="n"/>
+      <c r="T98" s="7" t="n"/>
+      <c r="U98" s="7" t="n"/>
+      <c r="V98" s="7" t="n"/>
+      <c r="W98" s="7" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="n"/>
@@ -3431,15 +3452,15 @@
       <c r="H99" s="7" t="n"/>
       <c r="I99" s="7" t="n"/>
       <c r="J99" s="7" t="n"/>
-      <c r="K99" s="7" t="n"/>
-      <c r="L99" s="7" t="n"/>
-      <c r="M99" s="7" t="n"/>
-      <c r="N99" s="7" t="n"/>
       <c r="O99" s="7" t="n"/>
       <c r="P99" s="7" t="n"/>
       <c r="Q99" s="7" t="n"/>
       <c r="R99" s="7" t="n"/>
       <c r="S99" s="7" t="n"/>
+      <c r="T99" s="7" t="n"/>
+      <c r="U99" s="7" t="n"/>
+      <c r="V99" s="7" t="n"/>
+      <c r="W99" s="7" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="n"/>
@@ -3452,15 +3473,15 @@
       <c r="H100" s="7" t="n"/>
       <c r="I100" s="7" t="n"/>
       <c r="J100" s="7" t="n"/>
-      <c r="K100" s="7" t="n"/>
-      <c r="L100" s="7" t="n"/>
-      <c r="M100" s="7" t="n"/>
-      <c r="N100" s="7" t="n"/>
       <c r="O100" s="7" t="n"/>
       <c r="P100" s="7" t="n"/>
       <c r="Q100" s="7" t="n"/>
       <c r="R100" s="7" t="n"/>
       <c r="S100" s="7" t="n"/>
+      <c r="T100" s="7" t="n"/>
+      <c r="U100" s="7" t="n"/>
+      <c r="V100" s="7" t="n"/>
+      <c r="W100" s="7" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="n"/>
@@ -3473,15 +3494,15 @@
       <c r="H101" s="7" t="n"/>
       <c r="I101" s="7" t="n"/>
       <c r="J101" s="7" t="n"/>
-      <c r="K101" s="7" t="n"/>
-      <c r="L101" s="7" t="n"/>
-      <c r="M101" s="7" t="n"/>
-      <c r="N101" s="7" t="n"/>
       <c r="O101" s="7" t="n"/>
       <c r="P101" s="7" t="n"/>
       <c r="Q101" s="7" t="n"/>
       <c r="R101" s="7" t="n"/>
       <c r="S101" s="7" t="n"/>
+      <c r="T101" s="7" t="n"/>
+      <c r="U101" s="7" t="n"/>
+      <c r="V101" s="7" t="n"/>
+      <c r="W101" s="7" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="n"/>
@@ -3494,15 +3515,15 @@
       <c r="H102" s="7" t="n"/>
       <c r="I102" s="7" t="n"/>
       <c r="J102" s="7" t="n"/>
-      <c r="K102" s="7" t="n"/>
-      <c r="L102" s="7" t="n"/>
-      <c r="M102" s="7" t="n"/>
-      <c r="N102" s="7" t="n"/>
       <c r="O102" s="7" t="n"/>
       <c r="P102" s="7" t="n"/>
       <c r="Q102" s="7" t="n"/>
       <c r="R102" s="7" t="n"/>
       <c r="S102" s="7" t="n"/>
+      <c r="T102" s="7" t="n"/>
+      <c r="U102" s="7" t="n"/>
+      <c r="V102" s="7" t="n"/>
+      <c r="W102" s="7" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="n"/>
@@ -3515,15 +3536,15 @@
       <c r="H103" s="7" t="n"/>
       <c r="I103" s="7" t="n"/>
       <c r="J103" s="7" t="n"/>
-      <c r="K103" s="7" t="n"/>
-      <c r="L103" s="7" t="n"/>
-      <c r="M103" s="7" t="n"/>
-      <c r="N103" s="7" t="n"/>
       <c r="O103" s="7" t="n"/>
       <c r="P103" s="7" t="n"/>
       <c r="Q103" s="7" t="n"/>
       <c r="R103" s="7" t="n"/>
       <c r="S103" s="7" t="n"/>
+      <c r="T103" s="7" t="n"/>
+      <c r="U103" s="7" t="n"/>
+      <c r="V103" s="7" t="n"/>
+      <c r="W103" s="7" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="n"/>
@@ -3536,15 +3557,15 @@
       <c r="H104" s="7" t="n"/>
       <c r="I104" s="7" t="n"/>
       <c r="J104" s="7" t="n"/>
-      <c r="K104" s="7" t="n"/>
-      <c r="L104" s="7" t="n"/>
-      <c r="M104" s="7" t="n"/>
-      <c r="N104" s="7" t="n"/>
       <c r="O104" s="7" t="n"/>
       <c r="P104" s="7" t="n"/>
       <c r="Q104" s="7" t="n"/>
       <c r="R104" s="7" t="n"/>
       <c r="S104" s="7" t="n"/>
+      <c r="T104" s="7" t="n"/>
+      <c r="U104" s="7" t="n"/>
+      <c r="V104" s="7" t="n"/>
+      <c r="W104" s="7" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="n"/>
@@ -3557,15 +3578,15 @@
       <c r="H105" s="7" t="n"/>
       <c r="I105" s="7" t="n"/>
       <c r="J105" s="7" t="n"/>
-      <c r="K105" s="7" t="n"/>
-      <c r="L105" s="7" t="n"/>
-      <c r="M105" s="7" t="n"/>
-      <c r="N105" s="7" t="n"/>
       <c r="O105" s="7" t="n"/>
       <c r="P105" s="7" t="n"/>
       <c r="Q105" s="7" t="n"/>
       <c r="R105" s="7" t="n"/>
       <c r="S105" s="7" t="n"/>
+      <c r="T105" s="7" t="n"/>
+      <c r="U105" s="7" t="n"/>
+      <c r="V105" s="7" t="n"/>
+      <c r="W105" s="7" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="n"/>
@@ -3578,15 +3599,15 @@
       <c r="H106" s="7" t="n"/>
       <c r="I106" s="7" t="n"/>
       <c r="J106" s="7" t="n"/>
-      <c r="K106" s="7" t="n"/>
-      <c r="L106" s="7" t="n"/>
-      <c r="M106" s="7" t="n"/>
-      <c r="N106" s="7" t="n"/>
       <c r="O106" s="7" t="n"/>
       <c r="P106" s="7" t="n"/>
       <c r="Q106" s="7" t="n"/>
       <c r="R106" s="7" t="n"/>
       <c r="S106" s="7" t="n"/>
+      <c r="T106" s="7" t="n"/>
+      <c r="U106" s="7" t="n"/>
+      <c r="V106" s="7" t="n"/>
+      <c r="W106" s="7" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="n"/>
@@ -3599,15 +3620,15 @@
       <c r="H107" s="7" t="n"/>
       <c r="I107" s="7" t="n"/>
       <c r="J107" s="7" t="n"/>
-      <c r="K107" s="7" t="n"/>
-      <c r="L107" s="7" t="n"/>
-      <c r="M107" s="7" t="n"/>
-      <c r="N107" s="7" t="n"/>
       <c r="O107" s="7" t="n"/>
       <c r="P107" s="7" t="n"/>
       <c r="Q107" s="7" t="n"/>
       <c r="R107" s="7" t="n"/>
       <c r="S107" s="7" t="n"/>
+      <c r="T107" s="7" t="n"/>
+      <c r="U107" s="7" t="n"/>
+      <c r="V107" s="7" t="n"/>
+      <c r="W107" s="7" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="n"/>
@@ -3620,15 +3641,15 @@
       <c r="H108" s="7" t="n"/>
       <c r="I108" s="7" t="n"/>
       <c r="J108" s="7" t="n"/>
-      <c r="K108" s="7" t="n"/>
-      <c r="L108" s="7" t="n"/>
-      <c r="M108" s="7" t="n"/>
-      <c r="N108" s="7" t="n"/>
       <c r="O108" s="7" t="n"/>
       <c r="P108" s="7" t="n"/>
       <c r="Q108" s="7" t="n"/>
       <c r="R108" s="7" t="n"/>
       <c r="S108" s="7" t="n"/>
+      <c r="T108" s="7" t="n"/>
+      <c r="U108" s="7" t="n"/>
+      <c r="V108" s="7" t="n"/>
+      <c r="W108" s="7" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="n"/>
@@ -3641,15 +3662,15 @@
       <c r="H109" s="7" t="n"/>
       <c r="I109" s="7" t="n"/>
       <c r="J109" s="7" t="n"/>
-      <c r="K109" s="7" t="n"/>
-      <c r="L109" s="7" t="n"/>
-      <c r="M109" s="7" t="n"/>
-      <c r="N109" s="7" t="n"/>
       <c r="O109" s="7" t="n"/>
       <c r="P109" s="7" t="n"/>
       <c r="Q109" s="7" t="n"/>
       <c r="R109" s="7" t="n"/>
       <c r="S109" s="7" t="n"/>
+      <c r="T109" s="7" t="n"/>
+      <c r="U109" s="7" t="n"/>
+      <c r="V109" s="7" t="n"/>
+      <c r="W109" s="7" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="n"/>
@@ -3662,15 +3683,15 @@
       <c r="H110" s="7" t="n"/>
       <c r="I110" s="7" t="n"/>
       <c r="J110" s="7" t="n"/>
-      <c r="K110" s="7" t="n"/>
-      <c r="L110" s="7" t="n"/>
-      <c r="M110" s="7" t="n"/>
-      <c r="N110" s="7" t="n"/>
       <c r="O110" s="7" t="n"/>
       <c r="P110" s="7" t="n"/>
       <c r="Q110" s="7" t="n"/>
       <c r="R110" s="7" t="n"/>
       <c r="S110" s="7" t="n"/>
+      <c r="T110" s="7" t="n"/>
+      <c r="U110" s="7" t="n"/>
+      <c r="V110" s="7" t="n"/>
+      <c r="W110" s="7" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="n"/>
@@ -3683,15 +3704,15 @@
       <c r="H111" s="7" t="n"/>
       <c r="I111" s="7" t="n"/>
       <c r="J111" s="7" t="n"/>
-      <c r="K111" s="7" t="n"/>
-      <c r="L111" s="7" t="n"/>
-      <c r="M111" s="7" t="n"/>
-      <c r="N111" s="7" t="n"/>
       <c r="O111" s="7" t="n"/>
       <c r="P111" s="7" t="n"/>
       <c r="Q111" s="7" t="n"/>
       <c r="R111" s="7" t="n"/>
       <c r="S111" s="7" t="n"/>
+      <c r="T111" s="7" t="n"/>
+      <c r="U111" s="7" t="n"/>
+      <c r="V111" s="7" t="n"/>
+      <c r="W111" s="7" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="n"/>
@@ -3704,15 +3725,15 @@
       <c r="H112" s="7" t="n"/>
       <c r="I112" s="7" t="n"/>
       <c r="J112" s="7" t="n"/>
-      <c r="K112" s="7" t="n"/>
-      <c r="L112" s="7" t="n"/>
-      <c r="M112" s="7" t="n"/>
-      <c r="N112" s="7" t="n"/>
       <c r="O112" s="7" t="n"/>
       <c r="P112" s="7" t="n"/>
       <c r="Q112" s="7" t="n"/>
       <c r="R112" s="7" t="n"/>
       <c r="S112" s="7" t="n"/>
+      <c r="T112" s="7" t="n"/>
+      <c r="U112" s="7" t="n"/>
+      <c r="V112" s="7" t="n"/>
+      <c r="W112" s="7" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="n"/>
@@ -3725,15 +3746,15 @@
       <c r="H113" s="7" t="n"/>
       <c r="I113" s="7" t="n"/>
       <c r="J113" s="7" t="n"/>
-      <c r="K113" s="7" t="n"/>
-      <c r="L113" s="7" t="n"/>
-      <c r="M113" s="7" t="n"/>
-      <c r="N113" s="7" t="n"/>
       <c r="O113" s="7" t="n"/>
       <c r="P113" s="7" t="n"/>
       <c r="Q113" s="7" t="n"/>
       <c r="R113" s="7" t="n"/>
       <c r="S113" s="7" t="n"/>
+      <c r="T113" s="7" t="n"/>
+      <c r="U113" s="7" t="n"/>
+      <c r="V113" s="7" t="n"/>
+      <c r="W113" s="7" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="n"/>
@@ -3746,15 +3767,15 @@
       <c r="H114" s="7" t="n"/>
       <c r="I114" s="7" t="n"/>
       <c r="J114" s="7" t="n"/>
-      <c r="K114" s="7" t="n"/>
-      <c r="L114" s="7" t="n"/>
-      <c r="M114" s="7" t="n"/>
-      <c r="N114" s="7" t="n"/>
       <c r="O114" s="7" t="n"/>
       <c r="P114" s="7" t="n"/>
       <c r="Q114" s="7" t="n"/>
       <c r="R114" s="7" t="n"/>
       <c r="S114" s="7" t="n"/>
+      <c r="T114" s="7" t="n"/>
+      <c r="U114" s="7" t="n"/>
+      <c r="V114" s="7" t="n"/>
+      <c r="W114" s="7" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="n"/>
@@ -3767,15 +3788,15 @@
       <c r="H115" s="7" t="n"/>
       <c r="I115" s="7" t="n"/>
       <c r="J115" s="7" t="n"/>
-      <c r="K115" s="7" t="n"/>
-      <c r="L115" s="7" t="n"/>
-      <c r="M115" s="7" t="n"/>
-      <c r="N115" s="7" t="n"/>
       <c r="O115" s="7" t="n"/>
       <c r="P115" s="7" t="n"/>
       <c r="Q115" s="7" t="n"/>
       <c r="R115" s="7" t="n"/>
       <c r="S115" s="7" t="n"/>
+      <c r="T115" s="7" t="n"/>
+      <c r="U115" s="7" t="n"/>
+      <c r="V115" s="7" t="n"/>
+      <c r="W115" s="7" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="n"/>
@@ -3788,15 +3809,15 @@
       <c r="H116" s="7" t="n"/>
       <c r="I116" s="7" t="n"/>
       <c r="J116" s="7" t="n"/>
-      <c r="K116" s="7" t="n"/>
-      <c r="L116" s="7" t="n"/>
-      <c r="M116" s="7" t="n"/>
-      <c r="N116" s="7" t="n"/>
       <c r="O116" s="7" t="n"/>
       <c r="P116" s="7" t="n"/>
       <c r="Q116" s="7" t="n"/>
       <c r="R116" s="7" t="n"/>
       <c r="S116" s="7" t="n"/>
+      <c r="T116" s="7" t="n"/>
+      <c r="U116" s="7" t="n"/>
+      <c r="V116" s="7" t="n"/>
+      <c r="W116" s="7" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="n"/>
@@ -3809,15 +3830,15 @@
       <c r="H117" s="7" t="n"/>
       <c r="I117" s="7" t="n"/>
       <c r="J117" s="7" t="n"/>
-      <c r="K117" s="7" t="n"/>
-      <c r="L117" s="7" t="n"/>
-      <c r="M117" s="7" t="n"/>
-      <c r="N117" s="7" t="n"/>
       <c r="O117" s="7" t="n"/>
       <c r="P117" s="7" t="n"/>
       <c r="Q117" s="7" t="n"/>
       <c r="R117" s="7" t="n"/>
       <c r="S117" s="7" t="n"/>
+      <c r="T117" s="7" t="n"/>
+      <c r="U117" s="7" t="n"/>
+      <c r="V117" s="7" t="n"/>
+      <c r="W117" s="7" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="n"/>
@@ -3830,15 +3851,15 @@
       <c r="H118" s="7" t="n"/>
       <c r="I118" s="7" t="n"/>
       <c r="J118" s="7" t="n"/>
-      <c r="K118" s="7" t="n"/>
-      <c r="L118" s="7" t="n"/>
-      <c r="M118" s="7" t="n"/>
-      <c r="N118" s="7" t="n"/>
       <c r="O118" s="7" t="n"/>
       <c r="P118" s="7" t="n"/>
       <c r="Q118" s="7" t="n"/>
       <c r="R118" s="7" t="n"/>
       <c r="S118" s="7" t="n"/>
+      <c r="T118" s="7" t="n"/>
+      <c r="U118" s="7" t="n"/>
+      <c r="V118" s="7" t="n"/>
+      <c r="W118" s="7" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="n"/>
@@ -3851,15 +3872,15 @@
       <c r="H119" s="7" t="n"/>
       <c r="I119" s="7" t="n"/>
       <c r="J119" s="7" t="n"/>
-      <c r="K119" s="7" t="n"/>
-      <c r="L119" s="7" t="n"/>
-      <c r="M119" s="7" t="n"/>
-      <c r="N119" s="7" t="n"/>
       <c r="O119" s="7" t="n"/>
       <c r="P119" s="7" t="n"/>
       <c r="Q119" s="7" t="n"/>
       <c r="R119" s="7" t="n"/>
       <c r="S119" s="7" t="n"/>
+      <c r="T119" s="7" t="n"/>
+      <c r="U119" s="7" t="n"/>
+      <c r="V119" s="7" t="n"/>
+      <c r="W119" s="7" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="n"/>
@@ -3872,15 +3893,15 @@
       <c r="H120" s="7" t="n"/>
       <c r="I120" s="7" t="n"/>
       <c r="J120" s="7" t="n"/>
-      <c r="K120" s="7" t="n"/>
-      <c r="L120" s="7" t="n"/>
-      <c r="M120" s="7" t="n"/>
-      <c r="N120" s="7" t="n"/>
       <c r="O120" s="7" t="n"/>
       <c r="P120" s="7" t="n"/>
       <c r="Q120" s="7" t="n"/>
       <c r="R120" s="7" t="n"/>
       <c r="S120" s="7" t="n"/>
+      <c r="T120" s="7" t="n"/>
+      <c r="U120" s="7" t="n"/>
+      <c r="V120" s="7" t="n"/>
+      <c r="W120" s="7" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="n"/>
@@ -3893,15 +3914,15 @@
       <c r="H121" s="7" t="n"/>
       <c r="I121" s="7" t="n"/>
       <c r="J121" s="7" t="n"/>
-      <c r="K121" s="7" t="n"/>
-      <c r="L121" s="7" t="n"/>
-      <c r="M121" s="7" t="n"/>
-      <c r="N121" s="7" t="n"/>
       <c r="O121" s="7" t="n"/>
       <c r="P121" s="7" t="n"/>
       <c r="Q121" s="7" t="n"/>
       <c r="R121" s="7" t="n"/>
       <c r="S121" s="7" t="n"/>
+      <c r="T121" s="7" t="n"/>
+      <c r="U121" s="7" t="n"/>
+      <c r="V121" s="7" t="n"/>
+      <c r="W121" s="7" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="n"/>
@@ -3914,15 +3935,15 @@
       <c r="H122" s="7" t="n"/>
       <c r="I122" s="7" t="n"/>
       <c r="J122" s="7" t="n"/>
-      <c r="K122" s="7" t="n"/>
-      <c r="L122" s="7" t="n"/>
-      <c r="M122" s="7" t="n"/>
-      <c r="N122" s="7" t="n"/>
       <c r="O122" s="7" t="n"/>
       <c r="P122" s="7" t="n"/>
       <c r="Q122" s="7" t="n"/>
       <c r="R122" s="7" t="n"/>
       <c r="S122" s="7" t="n"/>
+      <c r="T122" s="7" t="n"/>
+      <c r="U122" s="7" t="n"/>
+      <c r="V122" s="7" t="n"/>
+      <c r="W122" s="7" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="n"/>
@@ -3935,15 +3956,15 @@
       <c r="H123" s="7" t="n"/>
       <c r="I123" s="7" t="n"/>
       <c r="J123" s="7" t="n"/>
-      <c r="K123" s="7" t="n"/>
-      <c r="L123" s="7" t="n"/>
-      <c r="M123" s="7" t="n"/>
-      <c r="N123" s="7" t="n"/>
       <c r="O123" s="7" t="n"/>
       <c r="P123" s="7" t="n"/>
       <c r="Q123" s="7" t="n"/>
       <c r="R123" s="7" t="n"/>
       <c r="S123" s="7" t="n"/>
+      <c r="T123" s="7" t="n"/>
+      <c r="U123" s="7" t="n"/>
+      <c r="V123" s="7" t="n"/>
+      <c r="W123" s="7" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="n"/>
@@ -3956,15 +3977,15 @@
       <c r="H124" s="7" t="n"/>
       <c r="I124" s="7" t="n"/>
       <c r="J124" s="7" t="n"/>
-      <c r="K124" s="7" t="n"/>
-      <c r="L124" s="7" t="n"/>
-      <c r="M124" s="7" t="n"/>
-      <c r="N124" s="7" t="n"/>
       <c r="O124" s="7" t="n"/>
       <c r="P124" s="7" t="n"/>
       <c r="Q124" s="7" t="n"/>
       <c r="R124" s="7" t="n"/>
       <c r="S124" s="7" t="n"/>
+      <c r="T124" s="7" t="n"/>
+      <c r="U124" s="7" t="n"/>
+      <c r="V124" s="7" t="n"/>
+      <c r="W124" s="7" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="n"/>
@@ -3977,15 +3998,15 @@
       <c r="H125" s="7" t="n"/>
       <c r="I125" s="7" t="n"/>
       <c r="J125" s="7" t="n"/>
-      <c r="K125" s="7" t="n"/>
-      <c r="L125" s="7" t="n"/>
-      <c r="M125" s="7" t="n"/>
-      <c r="N125" s="7" t="n"/>
       <c r="O125" s="7" t="n"/>
       <c r="P125" s="7" t="n"/>
       <c r="Q125" s="7" t="n"/>
       <c r="R125" s="7" t="n"/>
       <c r="S125" s="7" t="n"/>
+      <c r="T125" s="7" t="n"/>
+      <c r="U125" s="7" t="n"/>
+      <c r="V125" s="7" t="n"/>
+      <c r="W125" s="7" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="n"/>
@@ -3998,15 +4019,15 @@
       <c r="H126" s="7" t="n"/>
       <c r="I126" s="7" t="n"/>
       <c r="J126" s="7" t="n"/>
-      <c r="K126" s="7" t="n"/>
-      <c r="L126" s="7" t="n"/>
-      <c r="M126" s="7" t="n"/>
-      <c r="N126" s="7" t="n"/>
       <c r="O126" s="7" t="n"/>
       <c r="P126" s="7" t="n"/>
       <c r="Q126" s="7" t="n"/>
       <c r="R126" s="7" t="n"/>
       <c r="S126" s="7" t="n"/>
+      <c r="T126" s="7" t="n"/>
+      <c r="U126" s="7" t="n"/>
+      <c r="V126" s="7" t="n"/>
+      <c r="W126" s="7" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="n"/>
@@ -4019,15 +4040,15 @@
       <c r="H127" s="7" t="n"/>
       <c r="I127" s="7" t="n"/>
       <c r="J127" s="7" t="n"/>
-      <c r="K127" s="7" t="n"/>
-      <c r="L127" s="7" t="n"/>
-      <c r="M127" s="7" t="n"/>
-      <c r="N127" s="7" t="n"/>
       <c r="O127" s="7" t="n"/>
       <c r="P127" s="7" t="n"/>
       <c r="Q127" s="7" t="n"/>
       <c r="R127" s="7" t="n"/>
       <c r="S127" s="7" t="n"/>
+      <c r="T127" s="7" t="n"/>
+      <c r="U127" s="7" t="n"/>
+      <c r="V127" s="7" t="n"/>
+      <c r="W127" s="7" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="n"/>
@@ -4040,15 +4061,15 @@
       <c r="H128" s="7" t="n"/>
       <c r="I128" s="7" t="n"/>
       <c r="J128" s="7" t="n"/>
-      <c r="K128" s="7" t="n"/>
-      <c r="L128" s="7" t="n"/>
-      <c r="M128" s="7" t="n"/>
-      <c r="N128" s="7" t="n"/>
       <c r="O128" s="7" t="n"/>
       <c r="P128" s="7" t="n"/>
       <c r="Q128" s="7" t="n"/>
       <c r="R128" s="7" t="n"/>
       <c r="S128" s="7" t="n"/>
+      <c r="T128" s="7" t="n"/>
+      <c r="U128" s="7" t="n"/>
+      <c r="V128" s="7" t="n"/>
+      <c r="W128" s="7" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="n"/>
@@ -4061,15 +4082,15 @@
       <c r="H129" s="7" t="n"/>
       <c r="I129" s="7" t="n"/>
       <c r="J129" s="7" t="n"/>
-      <c r="K129" s="7" t="n"/>
-      <c r="L129" s="7" t="n"/>
-      <c r="M129" s="7" t="n"/>
-      <c r="N129" s="7" t="n"/>
       <c r="O129" s="7" t="n"/>
       <c r="P129" s="7" t="n"/>
       <c r="Q129" s="7" t="n"/>
       <c r="R129" s="7" t="n"/>
       <c r="S129" s="7" t="n"/>
+      <c r="T129" s="7" t="n"/>
+      <c r="U129" s="7" t="n"/>
+      <c r="V129" s="7" t="n"/>
+      <c r="W129" s="7" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="n"/>
@@ -4082,15 +4103,15 @@
       <c r="H130" s="7" t="n"/>
       <c r="I130" s="7" t="n"/>
       <c r="J130" s="7" t="n"/>
-      <c r="K130" s="7" t="n"/>
-      <c r="L130" s="7" t="n"/>
-      <c r="M130" s="7" t="n"/>
-      <c r="N130" s="7" t="n"/>
       <c r="O130" s="7" t="n"/>
       <c r="P130" s="7" t="n"/>
       <c r="Q130" s="7" t="n"/>
       <c r="R130" s="7" t="n"/>
       <c r="S130" s="7" t="n"/>
+      <c r="T130" s="7" t="n"/>
+      <c r="U130" s="7" t="n"/>
+      <c r="V130" s="7" t="n"/>
+      <c r="W130" s="7" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="n"/>
@@ -4103,15 +4124,15 @@
       <c r="H131" s="7" t="n"/>
       <c r="I131" s="7" t="n"/>
       <c r="J131" s="7" t="n"/>
-      <c r="K131" s="7" t="n"/>
-      <c r="L131" s="7" t="n"/>
-      <c r="M131" s="7" t="n"/>
-      <c r="N131" s="7" t="n"/>
       <c r="O131" s="7" t="n"/>
       <c r="P131" s="7" t="n"/>
       <c r="Q131" s="7" t="n"/>
       <c r="R131" s="7" t="n"/>
       <c r="S131" s="7" t="n"/>
+      <c r="T131" s="7" t="n"/>
+      <c r="U131" s="7" t="n"/>
+      <c r="V131" s="7" t="n"/>
+      <c r="W131" s="7" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="n"/>
@@ -4124,15 +4145,15 @@
       <c r="H132" s="7" t="n"/>
       <c r="I132" s="7" t="n"/>
       <c r="J132" s="7" t="n"/>
-      <c r="K132" s="7" t="n"/>
-      <c r="L132" s="7" t="n"/>
-      <c r="M132" s="7" t="n"/>
-      <c r="N132" s="7" t="n"/>
       <c r="O132" s="7" t="n"/>
       <c r="P132" s="7" t="n"/>
       <c r="Q132" s="7" t="n"/>
       <c r="R132" s="7" t="n"/>
       <c r="S132" s="7" t="n"/>
+      <c r="T132" s="7" t="n"/>
+      <c r="U132" s="7" t="n"/>
+      <c r="V132" s="7" t="n"/>
+      <c r="W132" s="7" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="n"/>
@@ -4145,15 +4166,15 @@
       <c r="H133" s="7" t="n"/>
       <c r="I133" s="7" t="n"/>
       <c r="J133" s="7" t="n"/>
-      <c r="K133" s="7" t="n"/>
-      <c r="L133" s="7" t="n"/>
-      <c r="M133" s="7" t="n"/>
-      <c r="N133" s="7" t="n"/>
       <c r="O133" s="7" t="n"/>
       <c r="P133" s="7" t="n"/>
       <c r="Q133" s="7" t="n"/>
       <c r="R133" s="7" t="n"/>
       <c r="S133" s="7" t="n"/>
+      <c r="T133" s="7" t="n"/>
+      <c r="U133" s="7" t="n"/>
+      <c r="V133" s="7" t="n"/>
+      <c r="W133" s="7" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="n"/>
@@ -4166,15 +4187,15 @@
       <c r="H134" s="7" t="n"/>
       <c r="I134" s="7" t="n"/>
       <c r="J134" s="7" t="n"/>
-      <c r="K134" s="7" t="n"/>
-      <c r="L134" s="7" t="n"/>
-      <c r="M134" s="7" t="n"/>
-      <c r="N134" s="7" t="n"/>
       <c r="O134" s="7" t="n"/>
       <c r="P134" s="7" t="n"/>
       <c r="Q134" s="7" t="n"/>
       <c r="R134" s="7" t="n"/>
       <c r="S134" s="7" t="n"/>
+      <c r="T134" s="7" t="n"/>
+      <c r="U134" s="7" t="n"/>
+      <c r="V134" s="7" t="n"/>
+      <c r="W134" s="7" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="n"/>
@@ -4187,15 +4208,15 @@
       <c r="H135" s="7" t="n"/>
       <c r="I135" s="7" t="n"/>
       <c r="J135" s="7" t="n"/>
-      <c r="K135" s="7" t="n"/>
-      <c r="L135" s="7" t="n"/>
-      <c r="M135" s="7" t="n"/>
-      <c r="N135" s="7" t="n"/>
       <c r="O135" s="7" t="n"/>
       <c r="P135" s="7" t="n"/>
       <c r="Q135" s="7" t="n"/>
       <c r="R135" s="7" t="n"/>
       <c r="S135" s="7" t="n"/>
+      <c r="T135" s="7" t="n"/>
+      <c r="U135" s="7" t="n"/>
+      <c r="V135" s="7" t="n"/>
+      <c r="W135" s="7" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="n"/>
@@ -4208,15 +4229,15 @@
       <c r="H136" s="7" t="n"/>
       <c r="I136" s="7" t="n"/>
       <c r="J136" s="7" t="n"/>
-      <c r="K136" s="7" t="n"/>
-      <c r="L136" s="7" t="n"/>
-      <c r="M136" s="7" t="n"/>
-      <c r="N136" s="7" t="n"/>
       <c r="O136" s="7" t="n"/>
       <c r="P136" s="7" t="n"/>
       <c r="Q136" s="7" t="n"/>
       <c r="R136" s="7" t="n"/>
       <c r="S136" s="7" t="n"/>
+      <c r="T136" s="7" t="n"/>
+      <c r="U136" s="7" t="n"/>
+      <c r="V136" s="7" t="n"/>
+      <c r="W136" s="7" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="n"/>
@@ -4229,15 +4250,15 @@
       <c r="H137" s="7" t="n"/>
       <c r="I137" s="7" t="n"/>
       <c r="J137" s="7" t="n"/>
-      <c r="K137" s="7" t="n"/>
-      <c r="L137" s="7" t="n"/>
-      <c r="M137" s="7" t="n"/>
-      <c r="N137" s="7" t="n"/>
       <c r="O137" s="7" t="n"/>
       <c r="P137" s="7" t="n"/>
       <c r="Q137" s="7" t="n"/>
       <c r="R137" s="7" t="n"/>
       <c r="S137" s="7" t="n"/>
+      <c r="T137" s="7" t="n"/>
+      <c r="U137" s="7" t="n"/>
+      <c r="V137" s="7" t="n"/>
+      <c r="W137" s="7" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="n"/>
@@ -4250,15 +4271,15 @@
       <c r="H138" s="7" t="n"/>
       <c r="I138" s="7" t="n"/>
       <c r="J138" s="7" t="n"/>
-      <c r="K138" s="7" t="n"/>
-      <c r="L138" s="7" t="n"/>
-      <c r="M138" s="7" t="n"/>
-      <c r="N138" s="7" t="n"/>
       <c r="O138" s="7" t="n"/>
       <c r="P138" s="7" t="n"/>
       <c r="Q138" s="7" t="n"/>
       <c r="R138" s="7" t="n"/>
       <c r="S138" s="7" t="n"/>
+      <c r="T138" s="7" t="n"/>
+      <c r="U138" s="7" t="n"/>
+      <c r="V138" s="7" t="n"/>
+      <c r="W138" s="7" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="n"/>
@@ -4271,15 +4292,15 @@
       <c r="H139" s="7" t="n"/>
       <c r="I139" s="7" t="n"/>
       <c r="J139" s="7" t="n"/>
-      <c r="K139" s="7" t="n"/>
-      <c r="L139" s="7" t="n"/>
-      <c r="M139" s="7" t="n"/>
-      <c r="N139" s="7" t="n"/>
       <c r="O139" s="7" t="n"/>
       <c r="P139" s="7" t="n"/>
       <c r="Q139" s="7" t="n"/>
       <c r="R139" s="7" t="n"/>
       <c r="S139" s="7" t="n"/>
+      <c r="T139" s="7" t="n"/>
+      <c r="U139" s="7" t="n"/>
+      <c r="V139" s="7" t="n"/>
+      <c r="W139" s="7" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="n"/>
@@ -4292,15 +4313,15 @@
       <c r="H140" s="7" t="n"/>
       <c r="I140" s="7" t="n"/>
       <c r="J140" s="7" t="n"/>
-      <c r="K140" s="7" t="n"/>
-      <c r="L140" s="7" t="n"/>
-      <c r="M140" s="7" t="n"/>
-      <c r="N140" s="7" t="n"/>
       <c r="O140" s="7" t="n"/>
       <c r="P140" s="7" t="n"/>
       <c r="Q140" s="7" t="n"/>
       <c r="R140" s="7" t="n"/>
       <c r="S140" s="7" t="n"/>
+      <c r="T140" s="7" t="n"/>
+      <c r="U140" s="7" t="n"/>
+      <c r="V140" s="7" t="n"/>
+      <c r="W140" s="7" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="n"/>
@@ -4313,15 +4334,15 @@
       <c r="H141" s="7" t="n"/>
       <c r="I141" s="7" t="n"/>
       <c r="J141" s="7" t="n"/>
-      <c r="K141" s="7" t="n"/>
-      <c r="L141" s="7" t="n"/>
-      <c r="M141" s="7" t="n"/>
-      <c r="N141" s="7" t="n"/>
       <c r="O141" s="7" t="n"/>
       <c r="P141" s="7" t="n"/>
       <c r="Q141" s="7" t="n"/>
       <c r="R141" s="7" t="n"/>
       <c r="S141" s="7" t="n"/>
+      <c r="T141" s="7" t="n"/>
+      <c r="U141" s="7" t="n"/>
+      <c r="V141" s="7" t="n"/>
+      <c r="W141" s="7" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="n"/>
@@ -4334,15 +4355,15 @@
       <c r="H142" s="7" t="n"/>
       <c r="I142" s="7" t="n"/>
       <c r="J142" s="7" t="n"/>
-      <c r="K142" s="7" t="n"/>
-      <c r="L142" s="7" t="n"/>
-      <c r="M142" s="7" t="n"/>
-      <c r="N142" s="7" t="n"/>
       <c r="O142" s="7" t="n"/>
       <c r="P142" s="7" t="n"/>
       <c r="Q142" s="7" t="n"/>
       <c r="R142" s="7" t="n"/>
       <c r="S142" s="7" t="n"/>
+      <c r="T142" s="7" t="n"/>
+      <c r="U142" s="7" t="n"/>
+      <c r="V142" s="7" t="n"/>
+      <c r="W142" s="7" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="n"/>
@@ -4355,15 +4376,15 @@
       <c r="H143" s="7" t="n"/>
       <c r="I143" s="7" t="n"/>
       <c r="J143" s="7" t="n"/>
-      <c r="K143" s="7" t="n"/>
-      <c r="L143" s="7" t="n"/>
-      <c r="M143" s="7" t="n"/>
-      <c r="N143" s="7" t="n"/>
       <c r="O143" s="7" t="n"/>
       <c r="P143" s="7" t="n"/>
       <c r="Q143" s="7" t="n"/>
       <c r="R143" s="7" t="n"/>
       <c r="S143" s="7" t="n"/>
+      <c r="T143" s="7" t="n"/>
+      <c r="U143" s="7" t="n"/>
+      <c r="V143" s="7" t="n"/>
+      <c r="W143" s="7" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="n"/>
@@ -4376,15 +4397,15 @@
       <c r="H144" s="7" t="n"/>
       <c r="I144" s="7" t="n"/>
       <c r="J144" s="7" t="n"/>
-      <c r="K144" s="7" t="n"/>
-      <c r="L144" s="7" t="n"/>
-      <c r="M144" s="7" t="n"/>
-      <c r="N144" s="7" t="n"/>
       <c r="O144" s="7" t="n"/>
       <c r="P144" s="7" t="n"/>
       <c r="Q144" s="7" t="n"/>
       <c r="R144" s="7" t="n"/>
       <c r="S144" s="7" t="n"/>
+      <c r="T144" s="7" t="n"/>
+      <c r="U144" s="7" t="n"/>
+      <c r="V144" s="7" t="n"/>
+      <c r="W144" s="7" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="n"/>
@@ -4397,15 +4418,15 @@
       <c r="H145" s="7" t="n"/>
       <c r="I145" s="7" t="n"/>
       <c r="J145" s="7" t="n"/>
-      <c r="K145" s="7" t="n"/>
-      <c r="L145" s="7" t="n"/>
-      <c r="M145" s="7" t="n"/>
-      <c r="N145" s="7" t="n"/>
       <c r="O145" s="7" t="n"/>
       <c r="P145" s="7" t="n"/>
       <c r="Q145" s="7" t="n"/>
       <c r="R145" s="7" t="n"/>
       <c r="S145" s="7" t="n"/>
+      <c r="T145" s="7" t="n"/>
+      <c r="U145" s="7" t="n"/>
+      <c r="V145" s="7" t="n"/>
+      <c r="W145" s="7" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="n"/>
@@ -4418,15 +4439,15 @@
       <c r="H146" s="7" t="n"/>
       <c r="I146" s="7" t="n"/>
       <c r="J146" s="7" t="n"/>
-      <c r="K146" s="7" t="n"/>
-      <c r="L146" s="7" t="n"/>
-      <c r="M146" s="7" t="n"/>
-      <c r="N146" s="7" t="n"/>
       <c r="O146" s="7" t="n"/>
       <c r="P146" s="7" t="n"/>
       <c r="Q146" s="7" t="n"/>
       <c r="R146" s="7" t="n"/>
       <c r="S146" s="7" t="n"/>
+      <c r="T146" s="7" t="n"/>
+      <c r="U146" s="7" t="n"/>
+      <c r="V146" s="7" t="n"/>
+      <c r="W146" s="7" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="n"/>
@@ -4439,15 +4460,15 @@
       <c r="H147" s="7" t="n"/>
       <c r="I147" s="7" t="n"/>
       <c r="J147" s="7" t="n"/>
-      <c r="K147" s="7" t="n"/>
-      <c r="L147" s="7" t="n"/>
-      <c r="M147" s="7" t="n"/>
-      <c r="N147" s="7" t="n"/>
       <c r="O147" s="7" t="n"/>
       <c r="P147" s="7" t="n"/>
       <c r="Q147" s="7" t="n"/>
       <c r="R147" s="7" t="n"/>
       <c r="S147" s="7" t="n"/>
+      <c r="T147" s="7" t="n"/>
+      <c r="U147" s="7" t="n"/>
+      <c r="V147" s="7" t="n"/>
+      <c r="W147" s="7" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="n"/>
@@ -4460,15 +4481,15 @@
       <c r="H148" s="7" t="n"/>
       <c r="I148" s="7" t="n"/>
       <c r="J148" s="7" t="n"/>
-      <c r="K148" s="7" t="n"/>
-      <c r="L148" s="7" t="n"/>
-      <c r="M148" s="7" t="n"/>
-      <c r="N148" s="7" t="n"/>
       <c r="O148" s="7" t="n"/>
       <c r="P148" s="7" t="n"/>
       <c r="Q148" s="7" t="n"/>
       <c r="R148" s="7" t="n"/>
       <c r="S148" s="7" t="n"/>
+      <c r="T148" s="7" t="n"/>
+      <c r="U148" s="7" t="n"/>
+      <c r="V148" s="7" t="n"/>
+      <c r="W148" s="7" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="n"/>
@@ -4481,15 +4502,15 @@
       <c r="H149" s="7" t="n"/>
       <c r="I149" s="7" t="n"/>
       <c r="J149" s="7" t="n"/>
-      <c r="K149" s="7" t="n"/>
-      <c r="L149" s="7" t="n"/>
-      <c r="M149" s="7" t="n"/>
-      <c r="N149" s="7" t="n"/>
       <c r="O149" s="7" t="n"/>
       <c r="P149" s="7" t="n"/>
       <c r="Q149" s="7" t="n"/>
       <c r="R149" s="7" t="n"/>
       <c r="S149" s="7" t="n"/>
+      <c r="T149" s="7" t="n"/>
+      <c r="U149" s="7" t="n"/>
+      <c r="V149" s="7" t="n"/>
+      <c r="W149" s="7" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="n"/>
@@ -4502,15 +4523,15 @@
       <c r="H150" s="7" t="n"/>
       <c r="I150" s="7" t="n"/>
       <c r="J150" s="7" t="n"/>
-      <c r="K150" s="7" t="n"/>
-      <c r="L150" s="7" t="n"/>
-      <c r="M150" s="7" t="n"/>
-      <c r="N150" s="7" t="n"/>
       <c r="O150" s="7" t="n"/>
       <c r="P150" s="7" t="n"/>
       <c r="Q150" s="7" t="n"/>
       <c r="R150" s="7" t="n"/>
       <c r="S150" s="7" t="n"/>
+      <c r="T150" s="7" t="n"/>
+      <c r="U150" s="7" t="n"/>
+      <c r="V150" s="7" t="n"/>
+      <c r="W150" s="7" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="n"/>
@@ -4523,15 +4544,15 @@
       <c r="H151" s="7" t="n"/>
       <c r="I151" s="7" t="n"/>
       <c r="J151" s="7" t="n"/>
-      <c r="K151" s="7" t="n"/>
-      <c r="L151" s="7" t="n"/>
-      <c r="M151" s="7" t="n"/>
-      <c r="N151" s="7" t="n"/>
       <c r="O151" s="7" t="n"/>
       <c r="P151" s="7" t="n"/>
       <c r="Q151" s="7" t="n"/>
       <c r="R151" s="7" t="n"/>
       <c r="S151" s="7" t="n"/>
+      <c r="T151" s="7" t="n"/>
+      <c r="U151" s="7" t="n"/>
+      <c r="V151" s="7" t="n"/>
+      <c r="W151" s="7" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="n"/>
@@ -4544,15 +4565,15 @@
       <c r="H152" s="7" t="n"/>
       <c r="I152" s="7" t="n"/>
       <c r="J152" s="7" t="n"/>
-      <c r="K152" s="7" t="n"/>
-      <c r="L152" s="7" t="n"/>
-      <c r="M152" s="7" t="n"/>
-      <c r="N152" s="7" t="n"/>
       <c r="O152" s="7" t="n"/>
       <c r="P152" s="7" t="n"/>
       <c r="Q152" s="7" t="n"/>
       <c r="R152" s="7" t="n"/>
       <c r="S152" s="7" t="n"/>
+      <c r="T152" s="7" t="n"/>
+      <c r="U152" s="7" t="n"/>
+      <c r="V152" s="7" t="n"/>
+      <c r="W152" s="7" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="n"/>
@@ -4565,15 +4586,15 @@
       <c r="H153" s="7" t="n"/>
       <c r="I153" s="7" t="n"/>
       <c r="J153" s="7" t="n"/>
-      <c r="K153" s="7" t="n"/>
-      <c r="L153" s="7" t="n"/>
-      <c r="M153" s="7" t="n"/>
-      <c r="N153" s="7" t="n"/>
       <c r="O153" s="7" t="n"/>
       <c r="P153" s="7" t="n"/>
       <c r="Q153" s="7" t="n"/>
       <c r="R153" s="7" t="n"/>
       <c r="S153" s="7" t="n"/>
+      <c r="T153" s="7" t="n"/>
+      <c r="U153" s="7" t="n"/>
+      <c r="V153" s="7" t="n"/>
+      <c r="W153" s="7" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="n"/>
@@ -4586,15 +4607,15 @@
       <c r="H154" s="7" t="n"/>
       <c r="I154" s="7" t="n"/>
       <c r="J154" s="7" t="n"/>
-      <c r="K154" s="7" t="n"/>
-      <c r="L154" s="7" t="n"/>
-      <c r="M154" s="7" t="n"/>
-      <c r="N154" s="7" t="n"/>
       <c r="O154" s="7" t="n"/>
       <c r="P154" s="7" t="n"/>
       <c r="Q154" s="7" t="n"/>
       <c r="R154" s="7" t="n"/>
       <c r="S154" s="7" t="n"/>
+      <c r="T154" s="7" t="n"/>
+      <c r="U154" s="7" t="n"/>
+      <c r="V154" s="7" t="n"/>
+      <c r="W154" s="7" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="n"/>
@@ -4607,15 +4628,15 @@
       <c r="H155" s="7" t="n"/>
       <c r="I155" s="7" t="n"/>
       <c r="J155" s="7" t="n"/>
-      <c r="K155" s="7" t="n"/>
-      <c r="L155" s="7" t="n"/>
-      <c r="M155" s="7" t="n"/>
-      <c r="N155" s="7" t="n"/>
       <c r="O155" s="7" t="n"/>
       <c r="P155" s="7" t="n"/>
       <c r="Q155" s="7" t="n"/>
       <c r="R155" s="7" t="n"/>
       <c r="S155" s="7" t="n"/>
+      <c r="T155" s="7" t="n"/>
+      <c r="U155" s="7" t="n"/>
+      <c r="V155" s="7" t="n"/>
+      <c r="W155" s="7" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="n"/>
@@ -4628,15 +4649,15 @@
       <c r="H156" s="7" t="n"/>
       <c r="I156" s="7" t="n"/>
       <c r="J156" s="7" t="n"/>
-      <c r="K156" s="7" t="n"/>
-      <c r="L156" s="7" t="n"/>
-      <c r="M156" s="7" t="n"/>
-      <c r="N156" s="7" t="n"/>
       <c r="O156" s="7" t="n"/>
       <c r="P156" s="7" t="n"/>
       <c r="Q156" s="7" t="n"/>
       <c r="R156" s="7" t="n"/>
       <c r="S156" s="7" t="n"/>
+      <c r="T156" s="7" t="n"/>
+      <c r="U156" s="7" t="n"/>
+      <c r="V156" s="7" t="n"/>
+      <c r="W156" s="7" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="n"/>
@@ -4649,15 +4670,15 @@
       <c r="H157" s="7" t="n"/>
       <c r="I157" s="7" t="n"/>
       <c r="J157" s="7" t="n"/>
-      <c r="K157" s="7" t="n"/>
-      <c r="L157" s="7" t="n"/>
-      <c r="M157" s="7" t="n"/>
-      <c r="N157" s="7" t="n"/>
       <c r="O157" s="7" t="n"/>
       <c r="P157" s="7" t="n"/>
       <c r="Q157" s="7" t="n"/>
       <c r="R157" s="7" t="n"/>
       <c r="S157" s="7" t="n"/>
+      <c r="T157" s="7" t="n"/>
+      <c r="U157" s="7" t="n"/>
+      <c r="V157" s="7" t="n"/>
+      <c r="W157" s="7" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="n"/>
@@ -4670,15 +4691,15 @@
       <c r="H158" s="7" t="n"/>
       <c r="I158" s="7" t="n"/>
       <c r="J158" s="7" t="n"/>
-      <c r="K158" s="7" t="n"/>
-      <c r="L158" s="7" t="n"/>
-      <c r="M158" s="7" t="n"/>
-      <c r="N158" s="7" t="n"/>
       <c r="O158" s="7" t="n"/>
       <c r="P158" s="7" t="n"/>
       <c r="Q158" s="7" t="n"/>
       <c r="R158" s="7" t="n"/>
       <c r="S158" s="7" t="n"/>
+      <c r="T158" s="7" t="n"/>
+      <c r="U158" s="7" t="n"/>
+      <c r="V158" s="7" t="n"/>
+      <c r="W158" s="7" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="n"/>
@@ -4691,15 +4712,15 @@
       <c r="H159" s="7" t="n"/>
       <c r="I159" s="7" t="n"/>
       <c r="J159" s="7" t="n"/>
-      <c r="K159" s="7" t="n"/>
-      <c r="L159" s="7" t="n"/>
-      <c r="M159" s="7" t="n"/>
-      <c r="N159" s="7" t="n"/>
       <c r="O159" s="7" t="n"/>
       <c r="P159" s="7" t="n"/>
       <c r="Q159" s="7" t="n"/>
       <c r="R159" s="7" t="n"/>
       <c r="S159" s="7" t="n"/>
+      <c r="T159" s="7" t="n"/>
+      <c r="U159" s="7" t="n"/>
+      <c r="V159" s="7" t="n"/>
+      <c r="W159" s="7" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="n"/>
@@ -4712,15 +4733,15 @@
       <c r="H160" s="7" t="n"/>
       <c r="I160" s="7" t="n"/>
       <c r="J160" s="7" t="n"/>
-      <c r="K160" s="7" t="n"/>
-      <c r="L160" s="7" t="n"/>
-      <c r="M160" s="7" t="n"/>
-      <c r="N160" s="7" t="n"/>
       <c r="O160" s="7" t="n"/>
       <c r="P160" s="7" t="n"/>
       <c r="Q160" s="7" t="n"/>
       <c r="R160" s="7" t="n"/>
       <c r="S160" s="7" t="n"/>
+      <c r="T160" s="7" t="n"/>
+      <c r="U160" s="7" t="n"/>
+      <c r="V160" s="7" t="n"/>
+      <c r="W160" s="7" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="n"/>
@@ -4733,15 +4754,15 @@
       <c r="H161" s="7" t="n"/>
       <c r="I161" s="7" t="n"/>
       <c r="J161" s="7" t="n"/>
-      <c r="K161" s="7" t="n"/>
-      <c r="L161" s="7" t="n"/>
-      <c r="M161" s="7" t="n"/>
-      <c r="N161" s="7" t="n"/>
       <c r="O161" s="7" t="n"/>
       <c r="P161" s="7" t="n"/>
       <c r="Q161" s="7" t="n"/>
       <c r="R161" s="7" t="n"/>
       <c r="S161" s="7" t="n"/>
+      <c r="T161" s="7" t="n"/>
+      <c r="U161" s="7" t="n"/>
+      <c r="V161" s="7" t="n"/>
+      <c r="W161" s="7" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="n"/>
@@ -4754,15 +4775,15 @@
       <c r="H162" s="7" t="n"/>
       <c r="I162" s="7" t="n"/>
       <c r="J162" s="7" t="n"/>
-      <c r="K162" s="7" t="n"/>
-      <c r="L162" s="7" t="n"/>
-      <c r="M162" s="7" t="n"/>
-      <c r="N162" s="7" t="n"/>
       <c r="O162" s="7" t="n"/>
       <c r="P162" s="7" t="n"/>
       <c r="Q162" s="7" t="n"/>
       <c r="R162" s="7" t="n"/>
       <c r="S162" s="7" t="n"/>
+      <c r="T162" s="7" t="n"/>
+      <c r="U162" s="7" t="n"/>
+      <c r="V162" s="7" t="n"/>
+      <c r="W162" s="7" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="n"/>
@@ -4775,15 +4796,15 @@
       <c r="H163" s="7" t="n"/>
       <c r="I163" s="7" t="n"/>
       <c r="J163" s="7" t="n"/>
-      <c r="K163" s="7" t="n"/>
-      <c r="L163" s="7" t="n"/>
-      <c r="M163" s="7" t="n"/>
-      <c r="N163" s="7" t="n"/>
       <c r="O163" s="7" t="n"/>
       <c r="P163" s="7" t="n"/>
       <c r="Q163" s="7" t="n"/>
       <c r="R163" s="7" t="n"/>
       <c r="S163" s="7" t="n"/>
+      <c r="T163" s="7" t="n"/>
+      <c r="U163" s="7" t="n"/>
+      <c r="V163" s="7" t="n"/>
+      <c r="W163" s="7" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="n"/>
@@ -4796,15 +4817,15 @@
       <c r="H164" s="7" t="n"/>
       <c r="I164" s="7" t="n"/>
       <c r="J164" s="7" t="n"/>
-      <c r="K164" s="7" t="n"/>
-      <c r="L164" s="7" t="n"/>
-      <c r="M164" s="7" t="n"/>
-      <c r="N164" s="7" t="n"/>
       <c r="O164" s="7" t="n"/>
       <c r="P164" s="7" t="n"/>
       <c r="Q164" s="7" t="n"/>
       <c r="R164" s="7" t="n"/>
       <c r="S164" s="7" t="n"/>
+      <c r="T164" s="7" t="n"/>
+      <c r="U164" s="7" t="n"/>
+      <c r="V164" s="7" t="n"/>
+      <c r="W164" s="7" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="n"/>
@@ -4817,15 +4838,15 @@
       <c r="H165" s="7" t="n"/>
       <c r="I165" s="7" t="n"/>
       <c r="J165" s="7" t="n"/>
-      <c r="K165" s="7" t="n"/>
-      <c r="L165" s="7" t="n"/>
-      <c r="M165" s="7" t="n"/>
-      <c r="N165" s="7" t="n"/>
       <c r="O165" s="7" t="n"/>
       <c r="P165" s="7" t="n"/>
       <c r="Q165" s="7" t="n"/>
       <c r="R165" s="7" t="n"/>
       <c r="S165" s="7" t="n"/>
+      <c r="T165" s="7" t="n"/>
+      <c r="U165" s="7" t="n"/>
+      <c r="V165" s="7" t="n"/>
+      <c r="W165" s="7" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="n"/>
@@ -4838,15 +4859,15 @@
       <c r="H166" s="7" t="n"/>
       <c r="I166" s="7" t="n"/>
       <c r="J166" s="7" t="n"/>
-      <c r="K166" s="7" t="n"/>
-      <c r="L166" s="7" t="n"/>
-      <c r="M166" s="7" t="n"/>
-      <c r="N166" s="7" t="n"/>
       <c r="O166" s="7" t="n"/>
       <c r="P166" s="7" t="n"/>
       <c r="Q166" s="7" t="n"/>
       <c r="R166" s="7" t="n"/>
       <c r="S166" s="7" t="n"/>
+      <c r="T166" s="7" t="n"/>
+      <c r="U166" s="7" t="n"/>
+      <c r="V166" s="7" t="n"/>
+      <c r="W166" s="7" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="n"/>
@@ -4859,15 +4880,15 @@
       <c r="H167" s="7" t="n"/>
       <c r="I167" s="7" t="n"/>
       <c r="J167" s="7" t="n"/>
-      <c r="K167" s="7" t="n"/>
-      <c r="L167" s="7" t="n"/>
-      <c r="M167" s="7" t="n"/>
-      <c r="N167" s="7" t="n"/>
       <c r="O167" s="7" t="n"/>
       <c r="P167" s="7" t="n"/>
       <c r="Q167" s="7" t="n"/>
       <c r="R167" s="7" t="n"/>
       <c r="S167" s="7" t="n"/>
+      <c r="T167" s="7" t="n"/>
+      <c r="U167" s="7" t="n"/>
+      <c r="V167" s="7" t="n"/>
+      <c r="W167" s="7" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="n"/>
@@ -4880,15 +4901,15 @@
       <c r="H168" s="7" t="n"/>
       <c r="I168" s="7" t="n"/>
       <c r="J168" s="7" t="n"/>
-      <c r="K168" s="7" t="n"/>
-      <c r="L168" s="7" t="n"/>
-      <c r="M168" s="7" t="n"/>
-      <c r="N168" s="7" t="n"/>
       <c r="O168" s="7" t="n"/>
       <c r="P168" s="7" t="n"/>
       <c r="Q168" s="7" t="n"/>
       <c r="R168" s="7" t="n"/>
       <c r="S168" s="7" t="n"/>
+      <c r="T168" s="7" t="n"/>
+      <c r="U168" s="7" t="n"/>
+      <c r="V168" s="7" t="n"/>
+      <c r="W168" s="7" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="n"/>
@@ -4901,15 +4922,15 @@
       <c r="H169" s="7" t="n"/>
       <c r="I169" s="7" t="n"/>
       <c r="J169" s="7" t="n"/>
-      <c r="K169" s="7" t="n"/>
-      <c r="L169" s="7" t="n"/>
-      <c r="M169" s="7" t="n"/>
-      <c r="N169" s="7" t="n"/>
       <c r="O169" s="7" t="n"/>
       <c r="P169" s="7" t="n"/>
       <c r="Q169" s="7" t="n"/>
       <c r="R169" s="7" t="n"/>
       <c r="S169" s="7" t="n"/>
+      <c r="T169" s="7" t="n"/>
+      <c r="U169" s="7" t="n"/>
+      <c r="V169" s="7" t="n"/>
+      <c r="W169" s="7" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="n"/>
@@ -4922,15 +4943,15 @@
       <c r="H170" s="7" t="n"/>
       <c r="I170" s="7" t="n"/>
       <c r="J170" s="7" t="n"/>
-      <c r="K170" s="7" t="n"/>
-      <c r="L170" s="7" t="n"/>
-      <c r="M170" s="7" t="n"/>
-      <c r="N170" s="7" t="n"/>
       <c r="O170" s="7" t="n"/>
       <c r="P170" s="7" t="n"/>
       <c r="Q170" s="7" t="n"/>
       <c r="R170" s="7" t="n"/>
       <c r="S170" s="7" t="n"/>
+      <c r="T170" s="7" t="n"/>
+      <c r="U170" s="7" t="n"/>
+      <c r="V170" s="7" t="n"/>
+      <c r="W170" s="7" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="n"/>
@@ -4943,15 +4964,15 @@
       <c r="H171" s="7" t="n"/>
       <c r="I171" s="7" t="n"/>
       <c r="J171" s="7" t="n"/>
-      <c r="K171" s="7" t="n"/>
-      <c r="L171" s="7" t="n"/>
-      <c r="M171" s="7" t="n"/>
-      <c r="N171" s="7" t="n"/>
       <c r="O171" s="7" t="n"/>
       <c r="P171" s="7" t="n"/>
       <c r="Q171" s="7" t="n"/>
       <c r="R171" s="7" t="n"/>
       <c r="S171" s="7" t="n"/>
+      <c r="T171" s="7" t="n"/>
+      <c r="U171" s="7" t="n"/>
+      <c r="V171" s="7" t="n"/>
+      <c r="W171" s="7" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="n"/>
@@ -4964,15 +4985,15 @@
       <c r="H172" s="7" t="n"/>
       <c r="I172" s="7" t="n"/>
       <c r="J172" s="7" t="n"/>
-      <c r="K172" s="7" t="n"/>
-      <c r="L172" s="7" t="n"/>
-      <c r="M172" s="7" t="n"/>
-      <c r="N172" s="7" t="n"/>
       <c r="O172" s="7" t="n"/>
       <c r="P172" s="7" t="n"/>
       <c r="Q172" s="7" t="n"/>
       <c r="R172" s="7" t="n"/>
       <c r="S172" s="7" t="n"/>
+      <c r="T172" s="7" t="n"/>
+      <c r="U172" s="7" t="n"/>
+      <c r="V172" s="7" t="n"/>
+      <c r="W172" s="7" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="n"/>
@@ -4985,15 +5006,15 @@
       <c r="H173" s="7" t="n"/>
       <c r="I173" s="7" t="n"/>
       <c r="J173" s="7" t="n"/>
-      <c r="K173" s="7" t="n"/>
-      <c r="L173" s="7" t="n"/>
-      <c r="M173" s="7" t="n"/>
-      <c r="N173" s="7" t="n"/>
       <c r="O173" s="7" t="n"/>
       <c r="P173" s="7" t="n"/>
       <c r="Q173" s="7" t="n"/>
       <c r="R173" s="7" t="n"/>
       <c r="S173" s="7" t="n"/>
+      <c r="T173" s="7" t="n"/>
+      <c r="U173" s="7" t="n"/>
+      <c r="V173" s="7" t="n"/>
+      <c r="W173" s="7" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="n"/>
@@ -5006,15 +5027,15 @@
       <c r="H174" s="7" t="n"/>
       <c r="I174" s="7" t="n"/>
       <c r="J174" s="7" t="n"/>
-      <c r="K174" s="7" t="n"/>
-      <c r="L174" s="7" t="n"/>
-      <c r="M174" s="7" t="n"/>
-      <c r="N174" s="7" t="n"/>
       <c r="O174" s="7" t="n"/>
       <c r="P174" s="7" t="n"/>
       <c r="Q174" s="7" t="n"/>
       <c r="R174" s="7" t="n"/>
       <c r="S174" s="7" t="n"/>
+      <c r="T174" s="7" t="n"/>
+      <c r="U174" s="7" t="n"/>
+      <c r="V174" s="7" t="n"/>
+      <c r="W174" s="7" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="n"/>
@@ -5027,15 +5048,15 @@
       <c r="H175" s="7" t="n"/>
       <c r="I175" s="7" t="n"/>
       <c r="J175" s="7" t="n"/>
-      <c r="K175" s="7" t="n"/>
-      <c r="L175" s="7" t="n"/>
-      <c r="M175" s="7" t="n"/>
-      <c r="N175" s="7" t="n"/>
       <c r="O175" s="7" t="n"/>
       <c r="P175" s="7" t="n"/>
       <c r="Q175" s="7" t="n"/>
       <c r="R175" s="7" t="n"/>
       <c r="S175" s="7" t="n"/>
+      <c r="T175" s="7" t="n"/>
+      <c r="U175" s="7" t="n"/>
+      <c r="V175" s="7" t="n"/>
+      <c r="W175" s="7" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="n"/>
@@ -5048,15 +5069,15 @@
       <c r="H176" s="7" t="n"/>
       <c r="I176" s="7" t="n"/>
       <c r="J176" s="7" t="n"/>
-      <c r="K176" s="7" t="n"/>
-      <c r="L176" s="7" t="n"/>
-      <c r="M176" s="7" t="n"/>
-      <c r="N176" s="7" t="n"/>
       <c r="O176" s="7" t="n"/>
       <c r="P176" s="7" t="n"/>
       <c r="Q176" s="7" t="n"/>
       <c r="R176" s="7" t="n"/>
       <c r="S176" s="7" t="n"/>
+      <c r="T176" s="7" t="n"/>
+      <c r="U176" s="7" t="n"/>
+      <c r="V176" s="7" t="n"/>
+      <c r="W176" s="7" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="n"/>
@@ -5069,15 +5090,15 @@
       <c r="H177" s="7" t="n"/>
       <c r="I177" s="7" t="n"/>
       <c r="J177" s="7" t="n"/>
-      <c r="K177" s="7" t="n"/>
-      <c r="L177" s="7" t="n"/>
-      <c r="M177" s="7" t="n"/>
-      <c r="N177" s="7" t="n"/>
       <c r="O177" s="7" t="n"/>
       <c r="P177" s="7" t="n"/>
       <c r="Q177" s="7" t="n"/>
       <c r="R177" s="7" t="n"/>
       <c r="S177" s="7" t="n"/>
+      <c r="T177" s="7" t="n"/>
+      <c r="U177" s="7" t="n"/>
+      <c r="V177" s="7" t="n"/>
+      <c r="W177" s="7" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="n"/>
@@ -5090,15 +5111,15 @@
       <c r="H178" s="7" t="n"/>
       <c r="I178" s="7" t="n"/>
       <c r="J178" s="7" t="n"/>
-      <c r="K178" s="7" t="n"/>
-      <c r="L178" s="7" t="n"/>
-      <c r="M178" s="7" t="n"/>
-      <c r="N178" s="7" t="n"/>
       <c r="O178" s="7" t="n"/>
       <c r="P178" s="7" t="n"/>
       <c r="Q178" s="7" t="n"/>
       <c r="R178" s="7" t="n"/>
       <c r="S178" s="7" t="n"/>
+      <c r="T178" s="7" t="n"/>
+      <c r="U178" s="7" t="n"/>
+      <c r="V178" s="7" t="n"/>
+      <c r="W178" s="7" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="n"/>
@@ -5111,15 +5132,15 @@
       <c r="H179" s="7" t="n"/>
       <c r="I179" s="7" t="n"/>
       <c r="J179" s="7" t="n"/>
-      <c r="K179" s="7" t="n"/>
-      <c r="L179" s="7" t="n"/>
-      <c r="M179" s="7" t="n"/>
-      <c r="N179" s="7" t="n"/>
       <c r="O179" s="7" t="n"/>
       <c r="P179" s="7" t="n"/>
       <c r="Q179" s="7" t="n"/>
       <c r="R179" s="7" t="n"/>
       <c r="S179" s="7" t="n"/>
+      <c r="T179" s="7" t="n"/>
+      <c r="U179" s="7" t="n"/>
+      <c r="V179" s="7" t="n"/>
+      <c r="W179" s="7" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="n"/>
@@ -5132,15 +5153,15 @@
       <c r="H180" s="7" t="n"/>
       <c r="I180" s="7" t="n"/>
       <c r="J180" s="7" t="n"/>
-      <c r="K180" s="7" t="n"/>
-      <c r="L180" s="7" t="n"/>
-      <c r="M180" s="7" t="n"/>
-      <c r="N180" s="7" t="n"/>
       <c r="O180" s="7" t="n"/>
       <c r="P180" s="7" t="n"/>
       <c r="Q180" s="7" t="n"/>
       <c r="R180" s="7" t="n"/>
       <c r="S180" s="7" t="n"/>
+      <c r="T180" s="7" t="n"/>
+      <c r="U180" s="7" t="n"/>
+      <c r="V180" s="7" t="n"/>
+      <c r="W180" s="7" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="n"/>
@@ -5153,15 +5174,15 @@
       <c r="H181" s="7" t="n"/>
       <c r="I181" s="7" t="n"/>
       <c r="J181" s="7" t="n"/>
-      <c r="K181" s="7" t="n"/>
-      <c r="L181" s="7" t="n"/>
-      <c r="M181" s="7" t="n"/>
-      <c r="N181" s="7" t="n"/>
       <c r="O181" s="7" t="n"/>
       <c r="P181" s="7" t="n"/>
       <c r="Q181" s="7" t="n"/>
       <c r="R181" s="7" t="n"/>
       <c r="S181" s="7" t="n"/>
+      <c r="T181" s="7" t="n"/>
+      <c r="U181" s="7" t="n"/>
+      <c r="V181" s="7" t="n"/>
+      <c r="W181" s="7" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="n"/>
@@ -5174,15 +5195,15 @@
       <c r="H182" s="7" t="n"/>
       <c r="I182" s="7" t="n"/>
       <c r="J182" s="7" t="n"/>
-      <c r="K182" s="7" t="n"/>
-      <c r="L182" s="7" t="n"/>
-      <c r="M182" s="7" t="n"/>
-      <c r="N182" s="7" t="n"/>
       <c r="O182" s="7" t="n"/>
       <c r="P182" s="7" t="n"/>
       <c r="Q182" s="7" t="n"/>
       <c r="R182" s="7" t="n"/>
       <c r="S182" s="7" t="n"/>
+      <c r="T182" s="7" t="n"/>
+      <c r="U182" s="7" t="n"/>
+      <c r="V182" s="7" t="n"/>
+      <c r="W182" s="7" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="n"/>
@@ -5195,15 +5216,15 @@
       <c r="H183" s="7" t="n"/>
       <c r="I183" s="7" t="n"/>
       <c r="J183" s="7" t="n"/>
-      <c r="K183" s="7" t="n"/>
-      <c r="L183" s="7" t="n"/>
-      <c r="M183" s="7" t="n"/>
-      <c r="N183" s="7" t="n"/>
       <c r="O183" s="7" t="n"/>
       <c r="P183" s="7" t="n"/>
       <c r="Q183" s="7" t="n"/>
       <c r="R183" s="7" t="n"/>
       <c r="S183" s="7" t="n"/>
+      <c r="T183" s="7" t="n"/>
+      <c r="U183" s="7" t="n"/>
+      <c r="V183" s="7" t="n"/>
+      <c r="W183" s="7" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="n"/>
@@ -5216,15 +5237,15 @@
       <c r="H184" s="7" t="n"/>
       <c r="I184" s="7" t="n"/>
       <c r="J184" s="7" t="n"/>
-      <c r="K184" s="7" t="n"/>
-      <c r="L184" s="7" t="n"/>
-      <c r="M184" s="7" t="n"/>
-      <c r="N184" s="7" t="n"/>
       <c r="O184" s="7" t="n"/>
       <c r="P184" s="7" t="n"/>
       <c r="Q184" s="7" t="n"/>
       <c r="R184" s="7" t="n"/>
       <c r="S184" s="7" t="n"/>
+      <c r="T184" s="7" t="n"/>
+      <c r="U184" s="7" t="n"/>
+      <c r="V184" s="7" t="n"/>
+      <c r="W184" s="7" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="n"/>
@@ -5237,15 +5258,15 @@
       <c r="H185" s="7" t="n"/>
       <c r="I185" s="7" t="n"/>
       <c r="J185" s="7" t="n"/>
-      <c r="K185" s="7" t="n"/>
-      <c r="L185" s="7" t="n"/>
-      <c r="M185" s="7" t="n"/>
-      <c r="N185" s="7" t="n"/>
       <c r="O185" s="7" t="n"/>
       <c r="P185" s="7" t="n"/>
       <c r="Q185" s="7" t="n"/>
       <c r="R185" s="7" t="n"/>
       <c r="S185" s="7" t="n"/>
+      <c r="T185" s="7" t="n"/>
+      <c r="U185" s="7" t="n"/>
+      <c r="V185" s="7" t="n"/>
+      <c r="W185" s="7" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="n"/>
@@ -5258,15 +5279,15 @@
       <c r="H186" s="7" t="n"/>
       <c r="I186" s="7" t="n"/>
       <c r="J186" s="7" t="n"/>
-      <c r="K186" s="7" t="n"/>
-      <c r="L186" s="7" t="n"/>
-      <c r="M186" s="7" t="n"/>
-      <c r="N186" s="7" t="n"/>
       <c r="O186" s="7" t="n"/>
       <c r="P186" s="7" t="n"/>
       <c r="Q186" s="7" t="n"/>
       <c r="R186" s="7" t="n"/>
       <c r="S186" s="7" t="n"/>
+      <c r="T186" s="7" t="n"/>
+      <c r="U186" s="7" t="n"/>
+      <c r="V186" s="7" t="n"/>
+      <c r="W186" s="7" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="n"/>
@@ -5279,15 +5300,15 @@
       <c r="H187" s="7" t="n"/>
       <c r="I187" s="7" t="n"/>
       <c r="J187" s="7" t="n"/>
-      <c r="K187" s="7" t="n"/>
-      <c r="L187" s="7" t="n"/>
-      <c r="M187" s="7" t="n"/>
-      <c r="N187" s="7" t="n"/>
       <c r="O187" s="7" t="n"/>
       <c r="P187" s="7" t="n"/>
       <c r="Q187" s="7" t="n"/>
       <c r="R187" s="7" t="n"/>
       <c r="S187" s="7" t="n"/>
+      <c r="T187" s="7" t="n"/>
+      <c r="U187" s="7" t="n"/>
+      <c r="V187" s="7" t="n"/>
+      <c r="W187" s="7" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="n"/>
@@ -5300,15 +5321,15 @@
       <c r="H188" s="7" t="n"/>
       <c r="I188" s="7" t="n"/>
       <c r="J188" s="7" t="n"/>
-      <c r="K188" s="7" t="n"/>
-      <c r="L188" s="7" t="n"/>
-      <c r="M188" s="7" t="n"/>
-      <c r="N188" s="7" t="n"/>
       <c r="O188" s="7" t="n"/>
       <c r="P188" s="7" t="n"/>
       <c r="Q188" s="7" t="n"/>
       <c r="R188" s="7" t="n"/>
       <c r="S188" s="7" t="n"/>
+      <c r="T188" s="7" t="n"/>
+      <c r="U188" s="7" t="n"/>
+      <c r="V188" s="7" t="n"/>
+      <c r="W188" s="7" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="n"/>
@@ -5321,15 +5342,15 @@
       <c r="H189" s="7" t="n"/>
       <c r="I189" s="7" t="n"/>
       <c r="J189" s="7" t="n"/>
-      <c r="K189" s="7" t="n"/>
-      <c r="L189" s="7" t="n"/>
-      <c r="M189" s="7" t="n"/>
-      <c r="N189" s="7" t="n"/>
       <c r="O189" s="7" t="n"/>
       <c r="P189" s="7" t="n"/>
       <c r="Q189" s="7" t="n"/>
       <c r="R189" s="7" t="n"/>
       <c r="S189" s="7" t="n"/>
+      <c r="T189" s="7" t="n"/>
+      <c r="U189" s="7" t="n"/>
+      <c r="V189" s="7" t="n"/>
+      <c r="W189" s="7" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="n"/>
@@ -5342,15 +5363,15 @@
       <c r="H190" s="7" t="n"/>
       <c r="I190" s="7" t="n"/>
       <c r="J190" s="7" t="n"/>
-      <c r="K190" s="7" t="n"/>
-      <c r="L190" s="7" t="n"/>
-      <c r="M190" s="7" t="n"/>
-      <c r="N190" s="7" t="n"/>
       <c r="O190" s="7" t="n"/>
       <c r="P190" s="7" t="n"/>
       <c r="Q190" s="7" t="n"/>
       <c r="R190" s="7" t="n"/>
       <c r="S190" s="7" t="n"/>
+      <c r="T190" s="7" t="n"/>
+      <c r="U190" s="7" t="n"/>
+      <c r="V190" s="7" t="n"/>
+      <c r="W190" s="7" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="n"/>
@@ -5363,15 +5384,15 @@
       <c r="H191" s="7" t="n"/>
       <c r="I191" s="7" t="n"/>
       <c r="J191" s="7" t="n"/>
-      <c r="K191" s="7" t="n"/>
-      <c r="L191" s="7" t="n"/>
-      <c r="M191" s="7" t="n"/>
-      <c r="N191" s="7" t="n"/>
       <c r="O191" s="7" t="n"/>
       <c r="P191" s="7" t="n"/>
       <c r="Q191" s="7" t="n"/>
       <c r="R191" s="7" t="n"/>
       <c r="S191" s="7" t="n"/>
+      <c r="T191" s="7" t="n"/>
+      <c r="U191" s="7" t="n"/>
+      <c r="V191" s="7" t="n"/>
+      <c r="W191" s="7" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="n"/>
@@ -5384,15 +5405,15 @@
       <c r="H192" s="7" t="n"/>
       <c r="I192" s="7" t="n"/>
       <c r="J192" s="7" t="n"/>
-      <c r="K192" s="7" t="n"/>
-      <c r="L192" s="7" t="n"/>
-      <c r="M192" s="7" t="n"/>
-      <c r="N192" s="7" t="n"/>
       <c r="O192" s="7" t="n"/>
       <c r="P192" s="7" t="n"/>
       <c r="Q192" s="7" t="n"/>
       <c r="R192" s="7" t="n"/>
       <c r="S192" s="7" t="n"/>
+      <c r="T192" s="7" t="n"/>
+      <c r="U192" s="7" t="n"/>
+      <c r="V192" s="7" t="n"/>
+      <c r="W192" s="7" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="n"/>
@@ -5405,15 +5426,15 @@
       <c r="H193" s="7" t="n"/>
       <c r="I193" s="7" t="n"/>
       <c r="J193" s="7" t="n"/>
-      <c r="K193" s="7" t="n"/>
-      <c r="L193" s="7" t="n"/>
-      <c r="M193" s="7" t="n"/>
-      <c r="N193" s="7" t="n"/>
       <c r="O193" s="7" t="n"/>
       <c r="P193" s="7" t="n"/>
       <c r="Q193" s="7" t="n"/>
       <c r="R193" s="7" t="n"/>
       <c r="S193" s="7" t="n"/>
+      <c r="T193" s="7" t="n"/>
+      <c r="U193" s="7" t="n"/>
+      <c r="V193" s="7" t="n"/>
+      <c r="W193" s="7" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="n"/>
@@ -5426,15 +5447,15 @@
       <c r="H194" s="7" t="n"/>
       <c r="I194" s="7" t="n"/>
       <c r="J194" s="7" t="n"/>
-      <c r="K194" s="7" t="n"/>
-      <c r="L194" s="7" t="n"/>
-      <c r="M194" s="7" t="n"/>
-      <c r="N194" s="7" t="n"/>
       <c r="O194" s="7" t="n"/>
       <c r="P194" s="7" t="n"/>
       <c r="Q194" s="7" t="n"/>
       <c r="R194" s="7" t="n"/>
       <c r="S194" s="7" t="n"/>
+      <c r="T194" s="7" t="n"/>
+      <c r="U194" s="7" t="n"/>
+      <c r="V194" s="7" t="n"/>
+      <c r="W194" s="7" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="n"/>
@@ -5447,15 +5468,15 @@
       <c r="H195" s="7" t="n"/>
       <c r="I195" s="7" t="n"/>
       <c r="J195" s="7" t="n"/>
-      <c r="K195" s="7" t="n"/>
-      <c r="L195" s="7" t="n"/>
-      <c r="M195" s="7" t="n"/>
-      <c r="N195" s="7" t="n"/>
       <c r="O195" s="7" t="n"/>
       <c r="P195" s="7" t="n"/>
       <c r="Q195" s="7" t="n"/>
       <c r="R195" s="7" t="n"/>
       <c r="S195" s="7" t="n"/>
+      <c r="T195" s="7" t="n"/>
+      <c r="U195" s="7" t="n"/>
+      <c r="V195" s="7" t="n"/>
+      <c r="W195" s="7" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="n"/>
@@ -5468,15 +5489,15 @@
       <c r="H196" s="7" t="n"/>
       <c r="I196" s="7" t="n"/>
       <c r="J196" s="7" t="n"/>
-      <c r="K196" s="7" t="n"/>
-      <c r="L196" s="7" t="n"/>
-      <c r="M196" s="7" t="n"/>
-      <c r="N196" s="7" t="n"/>
       <c r="O196" s="7" t="n"/>
       <c r="P196" s="7" t="n"/>
       <c r="Q196" s="7" t="n"/>
       <c r="R196" s="7" t="n"/>
       <c r="S196" s="7" t="n"/>
+      <c r="T196" s="7" t="n"/>
+      <c r="U196" s="7" t="n"/>
+      <c r="V196" s="7" t="n"/>
+      <c r="W196" s="7" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="n"/>
@@ -5489,15 +5510,15 @@
       <c r="H197" s="7" t="n"/>
       <c r="I197" s="7" t="n"/>
       <c r="J197" s="7" t="n"/>
-      <c r="K197" s="7" t="n"/>
-      <c r="L197" s="7" t="n"/>
-      <c r="M197" s="7" t="n"/>
-      <c r="N197" s="7" t="n"/>
       <c r="O197" s="7" t="n"/>
       <c r="P197" s="7" t="n"/>
       <c r="Q197" s="7" t="n"/>
       <c r="R197" s="7" t="n"/>
       <c r="S197" s="7" t="n"/>
+      <c r="T197" s="7" t="n"/>
+      <c r="U197" s="7" t="n"/>
+      <c r="V197" s="7" t="n"/>
+      <c r="W197" s="7" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="n"/>
@@ -5510,15 +5531,15 @@
       <c r="H198" s="7" t="n"/>
       <c r="I198" s="7" t="n"/>
       <c r="J198" s="7" t="n"/>
-      <c r="K198" s="7" t="n"/>
-      <c r="L198" s="7" t="n"/>
-      <c r="M198" s="7" t="n"/>
-      <c r="N198" s="7" t="n"/>
       <c r="O198" s="7" t="n"/>
       <c r="P198" s="7" t="n"/>
       <c r="Q198" s="7" t="n"/>
       <c r="R198" s="7" t="n"/>
       <c r="S198" s="7" t="n"/>
+      <c r="T198" s="7" t="n"/>
+      <c r="U198" s="7" t="n"/>
+      <c r="V198" s="7" t="n"/>
+      <c r="W198" s="7" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="n"/>
@@ -5531,15 +5552,15 @@
       <c r="H199" s="7" t="n"/>
       <c r="I199" s="7" t="n"/>
       <c r="J199" s="7" t="n"/>
-      <c r="K199" s="7" t="n"/>
-      <c r="L199" s="7" t="n"/>
-      <c r="M199" s="7" t="n"/>
-      <c r="N199" s="7" t="n"/>
       <c r="O199" s="7" t="n"/>
       <c r="P199" s="7" t="n"/>
       <c r="Q199" s="7" t="n"/>
       <c r="R199" s="7" t="n"/>
       <c r="S199" s="7" t="n"/>
+      <c r="T199" s="7" t="n"/>
+      <c r="U199" s="7" t="n"/>
+      <c r="V199" s="7" t="n"/>
+      <c r="W199" s="7" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="n"/>
@@ -5552,15 +5573,15 @@
       <c r="H200" s="7" t="n"/>
       <c r="I200" s="7" t="n"/>
       <c r="J200" s="7" t="n"/>
-      <c r="K200" s="7" t="n"/>
-      <c r="L200" s="7" t="n"/>
-      <c r="M200" s="7" t="n"/>
-      <c r="N200" s="7" t="n"/>
       <c r="O200" s="7" t="n"/>
       <c r="P200" s="7" t="n"/>
       <c r="Q200" s="7" t="n"/>
       <c r="R200" s="7" t="n"/>
       <c r="S200" s="7" t="n"/>
+      <c r="T200" s="7" t="n"/>
+      <c r="U200" s="7" t="n"/>
+      <c r="V200" s="7" t="n"/>
+      <c r="W200" s="7" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="7" t="n"/>
@@ -5573,15 +5594,15 @@
       <c r="H201" s="7" t="n"/>
       <c r="I201" s="7" t="n"/>
       <c r="J201" s="7" t="n"/>
-      <c r="K201" s="7" t="n"/>
-      <c r="L201" s="7" t="n"/>
-      <c r="M201" s="7" t="n"/>
-      <c r="N201" s="7" t="n"/>
       <c r="O201" s="7" t="n"/>
       <c r="P201" s="7" t="n"/>
       <c r="Q201" s="7" t="n"/>
       <c r="R201" s="7" t="n"/>
       <c r="S201" s="7" t="n"/>
+      <c r="T201" s="7" t="n"/>
+      <c r="U201" s="7" t="n"/>
+      <c r="V201" s="7" t="n"/>
+      <c r="W201" s="7" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="7" t="n"/>
@@ -5594,15 +5615,15 @@
       <c r="H202" s="7" t="n"/>
       <c r="I202" s="7" t="n"/>
       <c r="J202" s="7" t="n"/>
-      <c r="K202" s="7" t="n"/>
-      <c r="L202" s="7" t="n"/>
-      <c r="M202" s="7" t="n"/>
-      <c r="N202" s="7" t="n"/>
       <c r="O202" s="7" t="n"/>
       <c r="P202" s="7" t="n"/>
       <c r="Q202" s="7" t="n"/>
       <c r="R202" s="7" t="n"/>
       <c r="S202" s="7" t="n"/>
+      <c r="T202" s="7" t="n"/>
+      <c r="U202" s="7" t="n"/>
+      <c r="V202" s="7" t="n"/>
+      <c r="W202" s="7" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="7" t="n"/>
@@ -5615,15 +5636,15 @@
       <c r="H203" s="7" t="n"/>
       <c r="I203" s="7" t="n"/>
       <c r="J203" s="7" t="n"/>
-      <c r="K203" s="7" t="n"/>
-      <c r="L203" s="7" t="n"/>
-      <c r="M203" s="7" t="n"/>
-      <c r="N203" s="7" t="n"/>
       <c r="O203" s="7" t="n"/>
       <c r="P203" s="7" t="n"/>
       <c r="Q203" s="7" t="n"/>
       <c r="R203" s="7" t="n"/>
       <c r="S203" s="7" t="n"/>
+      <c r="T203" s="7" t="n"/>
+      <c r="U203" s="7" t="n"/>
+      <c r="V203" s="7" t="n"/>
+      <c r="W203" s="7" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="7" t="n"/>
@@ -5636,15 +5657,15 @@
       <c r="H204" s="7" t="n"/>
       <c r="I204" s="7" t="n"/>
       <c r="J204" s="7" t="n"/>
-      <c r="K204" s="7" t="n"/>
-      <c r="L204" s="7" t="n"/>
-      <c r="M204" s="7" t="n"/>
-      <c r="N204" s="7" t="n"/>
       <c r="O204" s="7" t="n"/>
       <c r="P204" s="7" t="n"/>
       <c r="Q204" s="7" t="n"/>
       <c r="R204" s="7" t="n"/>
       <c r="S204" s="7" t="n"/>
+      <c r="T204" s="7" t="n"/>
+      <c r="U204" s="7" t="n"/>
+      <c r="V204" s="7" t="n"/>
+      <c r="W204" s="7" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="7" t="n"/>
@@ -5657,15 +5678,15 @@
       <c r="H205" s="7" t="n"/>
       <c r="I205" s="7" t="n"/>
       <c r="J205" s="7" t="n"/>
-      <c r="K205" s="7" t="n"/>
-      <c r="L205" s="7" t="n"/>
-      <c r="M205" s="7" t="n"/>
-      <c r="N205" s="7" t="n"/>
       <c r="O205" s="7" t="n"/>
       <c r="P205" s="7" t="n"/>
       <c r="Q205" s="7" t="n"/>
       <c r="R205" s="7" t="n"/>
       <c r="S205" s="7" t="n"/>
+      <c r="T205" s="7" t="n"/>
+      <c r="U205" s="7" t="n"/>
+      <c r="V205" s="7" t="n"/>
+      <c r="W205" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:S205"/>

</xml_diff>